<commit_message>
Fix investment workbook calculations
</commit_message>
<xml_diff>
--- a/final_report/宁波怡丰汇投资分析.xlsx
+++ b/final_report/宁波怡丰汇投资分析.xlsx
@@ -309,7 +309,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -331,11 +331,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -571,6 +615,8 @@
     <xf numFmtId="165" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1034,12 +1080,12 @@
           <t>宁波怡丰汇商业项目 – 主要参数汇总</t>
         </is>
       </c>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="6" t="n"/>
-      <c r="H1" s="6" t="n"/>
+      <c r="C1" s="81" t="n"/>
+      <c r="D1" s="81" t="n"/>
+      <c r="E1" s="81" t="n"/>
+      <c r="F1" s="81" t="n"/>
+      <c r="G1" s="81" t="n"/>
+      <c r="H1" s="82" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="6" t="n"/>
@@ -1056,12 +1102,12 @@
           <t>1. 项目面积（平方米）</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
+      <c r="C3" s="81" t="n"/>
+      <c r="D3" s="81" t="n"/>
+      <c r="E3" s="81" t="n"/>
+      <c r="F3" s="81" t="n"/>
+      <c r="G3" s="81" t="n"/>
+      <c r="H3" s="82" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="8" t="inlineStr">
@@ -1318,12 +1364,12 @@
           <t>2. 租金假设（首年平均日租金，元/天/平方米）</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
-      <c r="G15" s="6" t="n"/>
-      <c r="H15" s="6" t="n"/>
+      <c r="C15" s="81" t="n"/>
+      <c r="D15" s="81" t="n"/>
+      <c r="E15" s="81" t="n"/>
+      <c r="F15" s="81" t="n"/>
+      <c r="G15" s="81" t="n"/>
+      <c r="H15" s="82" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="9" t="inlineStr">
@@ -1460,12 +1506,12 @@
           <t>3. 租赁参数</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
+      <c r="C25" s="81" t="n"/>
+      <c r="D25" s="81" t="n"/>
+      <c r="E25" s="81" t="n"/>
+      <c r="F25" s="81" t="n"/>
+      <c r="G25" s="81" t="n"/>
+      <c r="H25" s="82" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="8" t="inlineStr">
@@ -1551,10 +1597,10 @@
         <v>0</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="G29" s="6" t="n"/>
       <c r="H29" s="6" t="n"/>
@@ -1595,12 +1641,12 @@
           <t>4. 停车费假设</t>
         </is>
       </c>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
+      <c r="C32" s="81" t="n"/>
+      <c r="D32" s="81" t="n"/>
+      <c r="E32" s="81" t="n"/>
+      <c r="F32" s="81" t="n"/>
+      <c r="G32" s="81" t="n"/>
+      <c r="H32" s="82" t="n"/>
     </row>
     <row r="33">
       <c r="B33" s="8" t="inlineStr">
@@ -1718,12 +1764,12 @@
           <t>5. 运营成本假设（首年全年基准，元）</t>
         </is>
       </c>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="6" t="n"/>
-      <c r="H39" s="6" t="n"/>
+      <c r="C39" s="81" t="n"/>
+      <c r="D39" s="81" t="n"/>
+      <c r="E39" s="81" t="n"/>
+      <c r="F39" s="81" t="n"/>
+      <c r="G39" s="81" t="n"/>
+      <c r="H39" s="82" t="n"/>
     </row>
     <row r="40">
       <c r="B40" s="16" t="inlineStr">
@@ -1875,12 +1921,12 @@
           <t>6. 费用增长率（相对上一年）</t>
         </is>
       </c>
-      <c r="C48" s="6" t="n"/>
-      <c r="D48" s="6" t="n"/>
-      <c r="E48" s="6" t="n"/>
-      <c r="F48" s="6" t="n"/>
-      <c r="G48" s="6" t="n"/>
-      <c r="H48" s="6" t="n"/>
+      <c r="C48" s="81" t="n"/>
+      <c r="D48" s="81" t="n"/>
+      <c r="E48" s="81" t="n"/>
+      <c r="F48" s="81" t="n"/>
+      <c r="G48" s="81" t="n"/>
+      <c r="H48" s="82" t="n"/>
     </row>
     <row r="49">
       <c r="B49" s="8" t="inlineStr">
@@ -2052,12 +2098,12 @@
           <t>7. 财务参数</t>
         </is>
       </c>
-      <c r="C57" s="6" t="n"/>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="6" t="n"/>
-      <c r="H57" s="6" t="n"/>
+      <c r="C57" s="81" t="n"/>
+      <c r="D57" s="81" t="n"/>
+      <c r="E57" s="81" t="n"/>
+      <c r="F57" s="81" t="n"/>
+      <c r="G57" s="81" t="n"/>
+      <c r="H57" s="82" t="n"/>
     </row>
     <row r="58">
       <c r="B58" s="16" t="inlineStr">
@@ -2240,11 +2286,11 @@
           <t>Step 1：年度经营现金流模型（万元）</t>
         </is>
       </c>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="6" t="n"/>
+      <c r="C1" s="81" t="n"/>
+      <c r="D1" s="81" t="n"/>
+      <c r="E1" s="81" t="n"/>
+      <c r="F1" s="81" t="n"/>
+      <c r="G1" s="82" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="18" t="inlineStr">
@@ -2252,11 +2298,11 @@
           <t>注：期初（Period 0）= 2026年1月1日；2026年为9个月运营期；所有金额单位为万元。</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
+      <c r="C2" s="81" t="n"/>
+      <c r="D2" s="81" t="n"/>
+      <c r="E2" s="81" t="n"/>
+      <c r="F2" s="81" t="n"/>
+      <c r="G2" s="82" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="6" t="n"/>
@@ -2308,11 +2354,11 @@
           <t>▶ 一、营业收入</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
+      <c r="C5" s="81" t="n"/>
+      <c r="D5" s="81" t="n"/>
+      <c r="E5" s="81" t="n"/>
+      <c r="F5" s="81" t="n"/>
+      <c r="G5" s="82" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="16" t="inlineStr">
@@ -2321,16 +2367,16 @@
         </is>
       </c>
       <c r="C6" s="21" t="n">
-        <v>2297.865452800001</v>
+        <v>2297.8654528</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>5412.940528250001</v>
+        <v>5412.94052825</v>
       </c>
       <c r="E6" s="21" t="n">
-        <v>5412.940528250001</v>
+        <v>5427.7705023</v>
       </c>
       <c r="F6" s="21" t="n">
-        <v>5575.328744097501</v>
+        <v>5575.3287440975</v>
       </c>
       <c r="G6" s="6" t="n"/>
     </row>
@@ -2347,7 +2393,7 @@
         <v>396.171</v>
       </c>
       <c r="E7" s="21" t="n">
-        <v>462.1995</v>
+        <v>463.4658</v>
       </c>
       <c r="F7" s="21" t="n">
         <v>528.228</v>
@@ -2384,13 +2430,13 @@
         <v>2997.5372248</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>6523.090792250001</v>
+        <v>6523.09079225</v>
       </c>
       <c r="E9" s="23" t="n">
-        <v>6589.11929225</v>
+        <v>6605.2155663</v>
       </c>
       <c r="F9" s="23" t="n">
-        <v>6817.536008097502</v>
+        <v>6817.5360080975</v>
       </c>
       <c r="G9" s="6" t="n"/>
     </row>
@@ -2400,11 +2446,11 @@
           <t>▶ 二、运营成本</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
+      <c r="C10" s="81" t="n"/>
+      <c r="D10" s="81" t="n"/>
+      <c r="E10" s="81" t="n"/>
+      <c r="F10" s="81" t="n"/>
+      <c r="G10" s="82" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="16" t="inlineStr">
@@ -2473,13 +2519,13 @@
         </is>
       </c>
       <c r="C14" s="21" t="n">
-        <v>57.44663632000001</v>
+        <v>57.44663632</v>
       </c>
       <c r="D14" s="21" t="n">
         <v>135.32351320625</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>135.32351320625</v>
+        <v>135.6942625575</v>
       </c>
       <c r="F14" s="21" t="n">
         <v>139.3832186024375</v>
@@ -2496,10 +2542,10 @@
         <v>240.8380425</v>
       </c>
       <c r="D15" s="21" t="n">
-        <v>330.7509117</v>
+        <v>330.7509117000001</v>
       </c>
       <c r="E15" s="21" t="n">
-        <v>340.673439051</v>
+        <v>340.6734390510001</v>
       </c>
       <c r="F15" s="21" t="n">
         <v>350.89364222253</v>
@@ -2513,16 +2559,16 @@
         </is>
       </c>
       <c r="C16" s="21" t="n">
-        <v>321.1173899999999</v>
+        <v>321.1173900000001</v>
       </c>
       <c r="D16" s="21" t="n">
-        <v>432.4380851999999</v>
+        <v>432.4380852</v>
       </c>
       <c r="E16" s="21" t="n">
-        <v>436.7624660519999</v>
+        <v>436.762466052</v>
       </c>
       <c r="F16" s="21" t="n">
-        <v>441.1300907125199</v>
+        <v>441.13009071252</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -2559,7 +2605,7 @@
         <v>2090.38796595625</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>2102.39113783475</v>
+        <v>2102.761887186</v>
       </c>
       <c r="F18" s="26" t="n">
         <v>2105.177622648752</v>
@@ -2572,11 +2618,11 @@
           <t>▶ 三、营业利润与税</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
-      <c r="G19" s="6" t="n"/>
+      <c r="C19" s="81" t="n"/>
+      <c r="D19" s="81" t="n"/>
+      <c r="E19" s="81" t="n"/>
+      <c r="F19" s="81" t="n"/>
+      <c r="G19" s="82" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="28" t="inlineStr">
@@ -2585,16 +2631,16 @@
         </is>
       </c>
       <c r="C20" s="29" t="n">
-        <v>1470.216134730001</v>
+        <v>1470.21613473</v>
       </c>
       <c r="D20" s="29" t="n">
-        <v>4432.702826293751</v>
+        <v>4432.70282629375</v>
       </c>
       <c r="E20" s="29" t="n">
-        <v>4486.72815441525</v>
+        <v>4502.453679114001</v>
       </c>
       <c r="F20" s="29" t="n">
-        <v>4712.358385448749</v>
+        <v>4712.358385448747</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -2605,13 +2651,13 @@
         </is>
       </c>
       <c r="C21" s="21" t="n">
-        <v>367.5540336825002</v>
+        <v>367.5540336825001</v>
       </c>
       <c r="D21" s="21" t="n">
         <v>1108.175706573438</v>
       </c>
       <c r="E21" s="21" t="n">
-        <v>1121.682038603813</v>
+        <v>1125.6134197785</v>
       </c>
       <c r="F21" s="21" t="n">
         <v>1178.089596362187</v>
@@ -2628,13 +2674,13 @@
         <v>1102.6621010475</v>
       </c>
       <c r="D22" s="31" t="n">
-        <v>3324.527119720313</v>
+        <v>3324.527119720312</v>
       </c>
       <c r="E22" s="31" t="n">
-        <v>3365.046115811438</v>
+        <v>3376.8402593355</v>
       </c>
       <c r="F22" s="31" t="n">
-        <v>3534.268789086562</v>
+        <v>3534.26878908656</v>
       </c>
       <c r="G22" s="6" t="n"/>
     </row>
@@ -2644,11 +2690,11 @@
           <t>▶ 四、退出价值（永续年金 i=8%）</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n"/>
+      <c r="C23" s="81" t="n"/>
+      <c r="D23" s="81" t="n"/>
+      <c r="E23" s="81" t="n"/>
+      <c r="F23" s="81" t="n"/>
+      <c r="G23" s="82" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="32" t="inlineStr">
@@ -2660,7 +2706,7 @@
       <c r="D24" s="33" t="n"/>
       <c r="E24" s="33" t="n"/>
       <c r="F24" s="33" t="n">
-        <v>44178.35986358202</v>
+        <v>44178.359863582</v>
       </c>
       <c r="G24" s="6" t="n"/>
     </row>
@@ -2670,11 +2716,11 @@
           <t>▶ 五、年度总现金流</t>
         </is>
       </c>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
+      <c r="C25" s="81" t="n"/>
+      <c r="D25" s="81" t="n"/>
+      <c r="E25" s="81" t="n"/>
+      <c r="F25" s="81" t="n"/>
+      <c r="G25" s="82" t="n"/>
     </row>
     <row r="26">
       <c r="B26" s="22" t="inlineStr">
@@ -2686,13 +2732,13 @@
         <v>1102.6621010475</v>
       </c>
       <c r="D26" s="23" t="n">
-        <v>3324.527119720313</v>
+        <v>3324.527119720312</v>
       </c>
       <c r="E26" s="23" t="n">
-        <v>3365.046115811438</v>
+        <v>3376.8402593355</v>
       </c>
       <c r="F26" s="23" t="n">
-        <v>47712.62865266858</v>
+        <v>47712.62865266857</v>
       </c>
       <c r="G26" s="6" t="n"/>
     </row>
@@ -2710,11 +2756,11 @@
           <t>关键运营指标</t>
         </is>
       </c>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
+      <c r="C28" s="81" t="n"/>
+      <c r="D28" s="81" t="n"/>
+      <c r="E28" s="81" t="n"/>
+      <c r="F28" s="81" t="n"/>
+      <c r="G28" s="82" t="n"/>
     </row>
     <row r="29">
       <c r="B29" s="16" t="inlineStr">
@@ -2723,16 +2769,16 @@
         </is>
       </c>
       <c r="C29" s="35" t="n">
-        <v>8.000000000000001e-05</v>
+        <v>0.8</v>
       </c>
       <c r="D29" s="35" t="n">
-        <v>9.499999999999999e-05</v>
+        <v>0.95</v>
       </c>
       <c r="E29" s="35" t="n">
-        <v>9.499999999999999e-05</v>
+        <v>0.95</v>
       </c>
       <c r="F29" s="35" t="n">
-        <v>9.499999999999999e-05</v>
+        <v>0.95</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -2743,16 +2789,16 @@
         </is>
       </c>
       <c r="C30" s="10" t="n">
-        <v>0.0275</v>
+        <v>275</v>
       </c>
       <c r="D30" s="10" t="n">
-        <v>0.0365</v>
+        <v>365</v>
       </c>
       <c r="E30" s="10" t="n">
-        <v>0.0365</v>
+        <v>366</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>0.0365</v>
+        <v>365</v>
       </c>
       <c r="G30" s="6" t="n"/>
     </row>
@@ -2763,16 +2809,16 @@
         </is>
       </c>
       <c r="C31" s="35" t="n">
-        <v>7.66584459331716e-05</v>
+        <v>0.7665844593317158</v>
       </c>
       <c r="D31" s="35" t="n">
-        <v>8.298122317538559e-05</v>
+        <v>0.8298122317538558</v>
       </c>
       <c r="E31" s="35" t="n">
-        <v>8.214968174300016e-05</v>
+        <v>0.8217401003523097</v>
       </c>
       <c r="F31" s="35" t="n">
-        <v>8.177923427871046e-05</v>
+        <v>0.8177923427871048</v>
       </c>
       <c r="G31" s="6" t="n"/>
     </row>
@@ -2783,16 +2829,16 @@
         </is>
       </c>
       <c r="C32" s="35" t="n">
-        <v>4.904746878758429e-05</v>
+        <v>0.4904746878758428</v>
       </c>
       <c r="D32" s="35" t="n">
-        <v>6.795402620426788e-05</v>
+        <v>0.6795402620426788</v>
       </c>
       <c r="E32" s="35" t="n">
-        <v>6.809298717193443e-05</v>
+        <v>0.6816512850974386</v>
       </c>
       <c r="F32" s="35" t="n">
-        <v>6.912113672522835e-05</v>
+        <v>0.6912113672522834</v>
       </c>
       <c r="G32" s="6" t="n"/>
     </row>
@@ -2850,10 +2896,10 @@
           <t>Step 1（补充）：2026年季度现金流分析（万元）</t>
         </is>
       </c>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
+      <c r="C1" s="81" t="n"/>
+      <c r="D1" s="81" t="n"/>
+      <c r="E1" s="81" t="n"/>
+      <c r="F1" s="82" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="18" t="inlineStr">
@@ -2861,10 +2907,10 @@
           <t>说明：Q1为收购期无运营；Q2免租期仅有停车费+物业费；Q3起租金开始收取。税收按年度汇总计算。</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
+      <c r="C2" s="81" t="n"/>
+      <c r="D2" s="81" t="n"/>
+      <c r="E2" s="81" t="n"/>
+      <c r="F2" s="82" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="6" t="n"/>
@@ -2906,10 +2952,10 @@
           <t>收入</t>
         </is>
       </c>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
+      <c r="C5" s="81" t="n"/>
+      <c r="D5" s="81" t="n"/>
+      <c r="E5" s="81" t="n"/>
+      <c r="F5" s="82" t="n"/>
     </row>
     <row r="6">
       <c r="B6" s="36" t="inlineStr">
@@ -2993,10 +3039,10 @@
           <t>运营成本</t>
         </is>
       </c>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
+      <c r="C10" s="81" t="n"/>
+      <c r="D10" s="81" t="n"/>
+      <c r="E10" s="81" t="n"/>
+      <c r="F10" s="82" t="n"/>
     </row>
     <row r="11">
       <c r="B11" s="38" t="inlineStr">
@@ -3008,13 +3054,13 @@
         <v>0</v>
       </c>
       <c r="D11" s="39" t="n">
-        <v>488.6158001506849</v>
+        <v>509.1070300233333</v>
       </c>
       <c r="E11" s="39" t="n">
-        <v>522.7085227079452</v>
+        <v>509.1070300233333</v>
       </c>
       <c r="F11" s="39" t="n">
-        <v>522.7085227079452</v>
+        <v>509.1070300233333</v>
       </c>
     </row>
     <row r="12">
@@ -3023,10 +3069,10 @@
           <t>利润（税前，季度口径）</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
+      <c r="C12" s="81" t="n"/>
+      <c r="D12" s="81" t="n"/>
+      <c r="E12" s="81" t="n"/>
+      <c r="F12" s="82" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="30" t="inlineStr">
@@ -3038,13 +3084,13 @@
         <v>0</v>
       </c>
       <c r="D13" s="31" t="n">
-        <v>-255.9948761506849</v>
+        <v>-276.4861060233333</v>
       </c>
       <c r="E13" s="31" t="n">
-        <v>859.7496276920549</v>
+        <v>873.3511203766666</v>
       </c>
       <c r="F13" s="31" t="n">
-        <v>859.7496276920549</v>
+        <v>873.3511203766666</v>
       </c>
     </row>
     <row r="14">
@@ -3060,10 +3106,10 @@
           <t>2026全年汇总（与年度现金流匹配）</t>
         </is>
       </c>
-      <c r="C15" s="6" t="n"/>
-      <c r="D15" s="6" t="n"/>
-      <c r="E15" s="6" t="n"/>
-      <c r="F15" s="6" t="n"/>
+      <c r="C15" s="81" t="n"/>
+      <c r="D15" s="81" t="n"/>
+      <c r="E15" s="81" t="n"/>
+      <c r="F15" s="82" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="32" t="inlineStr">
@@ -3110,10 +3156,10 @@
           <t>季度现金流改善分析</t>
         </is>
       </c>
-      <c r="C19" s="6" t="n"/>
-      <c r="D19" s="6" t="n"/>
-      <c r="E19" s="6" t="n"/>
-      <c r="F19" s="6" t="n"/>
+      <c r="C19" s="81" t="n"/>
+      <c r="D19" s="81" t="n"/>
+      <c r="E19" s="81" t="n"/>
+      <c r="F19" s="82" t="n"/>
     </row>
     <row r="20">
       <c r="B20" s="41" t="inlineStr">
@@ -3129,7 +3175,7 @@
     <row r="21">
       <c r="B21" s="41" t="inlineStr">
         <is>
-          <t>Q2 → Q3：免租期结束，租金收入涌入，季度税前利润大幅转正（约+1116万元）</t>
+          <t>Q2 → Q3：免租期结束，租金收入开始确认，季度税前利润大幅转正（约+1150万元）</t>
         </is>
       </c>
       <c r="C21" s="6" t="n"/>
@@ -3151,7 +3197,7 @@
     <row r="23">
       <c r="B23" s="42" t="inlineStr">
         <is>
-          <t>改造期年度净CF（2026）≈ 1103万元  vs  稳定期（2027）≈ 3325万元，相差约2222万元（202%增幅）</t>
+          <t>改造期年度净CF（2026）≈ 1103万元  vs  稳定期（2027）≈ 3325万元，相差约2222万元（约202%增幅）</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>
@@ -3204,11 +3250,11 @@
           <t>Step 2：收购价格估算（MARR = 12%）</t>
         </is>
       </c>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="6" t="n"/>
+      <c r="C1" s="81" t="n"/>
+      <c r="D1" s="81" t="n"/>
+      <c r="E1" s="81" t="n"/>
+      <c r="F1" s="81" t="n"/>
+      <c r="G1" s="82" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="6" t="n"/>
@@ -3224,11 +3270,11 @@
           <t>一、未来现金流现值计算（折现率12%）</t>
         </is>
       </c>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
+      <c r="C3" s="81" t="n"/>
+      <c r="D3" s="81" t="n"/>
+      <c r="E3" s="81" t="n"/>
+      <c r="F3" s="81" t="n"/>
+      <c r="G3" s="82" t="n"/>
     </row>
     <row r="4">
       <c r="B4" s="8" t="inlineStr">
@@ -3264,16 +3310,14 @@
           <t>2026年</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
-        <is>
-          <t>改造期（9个月运营）</t>
-        </is>
+      <c r="C5" s="16" t="n">
+        <v>1102.6621010475</v>
       </c>
       <c r="D5" s="21" t="n">
-        <v>1102.6621010475</v>
+        <v>0.8928571428571428</v>
       </c>
       <c r="E5" s="43" t="n">
-        <v>0.8928571428571428</v>
+        <v>984.5197330781251</v>
       </c>
       <c r="F5" s="29" t="n">
         <v>984.5197330781253</v>
@@ -3286,16 +3330,14 @@
           <t>2027年</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>稳定期</t>
-        </is>
+      <c r="C6" s="16" t="n">
+        <v>3324.527119720312</v>
       </c>
       <c r="D6" s="21" t="n">
-        <v>3324.527119720313</v>
+        <v>0.7971938775510203</v>
       </c>
       <c r="E6" s="43" t="n">
-        <v>0.7971938775510203</v>
+        <v>2650.292665593361</v>
       </c>
       <c r="F6" s="29" t="n">
         <v>2650.292665593362</v>
@@ -3308,16 +3350,14 @@
           <t>2028年</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
-        <is>
-          <t>稳定期</t>
-        </is>
+      <c r="C7" s="16" t="n">
+        <v>3376.8402593355</v>
       </c>
       <c r="D7" s="21" t="n">
-        <v>3365.046115811438</v>
+        <v>0.7117802478134109</v>
       </c>
       <c r="E7" s="43" t="n">
-        <v>0.7117802478134109</v>
+        <v>2403.568196616125</v>
       </c>
       <c r="F7" s="29" t="n">
         <v>2395.173358215821</v>
@@ -3330,16 +3370,14 @@
           <t>2029年</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>稳定期 + 退出价值</t>
-        </is>
+      <c r="C8" s="16" t="n">
+        <v>47712.62865266857</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>47712.62865266858</v>
+        <v>0.6355180784048311</v>
       </c>
       <c r="E8" s="43" t="n">
-        <v>0.6355180784048311</v>
+        <v>30322.23807698721</v>
       </c>
       <c r="F8" s="29" t="n">
         <v>30322.23807698723</v>
@@ -3356,7 +3394,7 @@
       <c r="D9" s="6" t="n"/>
       <c r="E9" s="6" t="n"/>
       <c r="F9" s="44" t="n">
-        <v>36352.22383387454</v>
+        <v>36360.61867227482</v>
       </c>
       <c r="G9" s="6" t="n"/>
     </row>
@@ -3374,11 +3412,11 @@
           <t>二、收购价格推算</t>
         </is>
       </c>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
-      <c r="E11" s="6" t="n"/>
-      <c r="F11" s="6" t="n"/>
-      <c r="G11" s="6" t="n"/>
+      <c r="C11" s="81" t="n"/>
+      <c r="D11" s="81" t="n"/>
+      <c r="E11" s="81" t="n"/>
+      <c r="F11" s="81" t="n"/>
+      <c r="G11" s="82" t="n"/>
     </row>
     <row r="12">
       <c r="B12" s="16" t="inlineStr">
@@ -3387,7 +3425,7 @@
         </is>
       </c>
       <c r="C12" s="21" t="n">
-        <v>36352.22383387454</v>
+        <v>36360.61867227482</v>
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
@@ -3441,7 +3479,7 @@
         </is>
       </c>
       <c r="C15" s="31" t="n">
-        <v>34252.22383387454</v>
+        <v>34260.61867227482</v>
       </c>
       <c r="D15" s="45" t="inlineStr">
         <is>
@@ -3477,7 +3515,7 @@
         </is>
       </c>
       <c r="C17" s="31" t="n">
-        <v>33254.58624648013</v>
+        <v>33262.73657502409</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
@@ -3495,7 +3533,7 @@
         </is>
       </c>
       <c r="C18" s="21" t="n">
-        <v>997.6375873944039</v>
+        <v>997.8820972507227</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
@@ -3549,7 +3587,7 @@
         </is>
       </c>
       <c r="C21" s="31" t="n">
-        <v>36352.22383387454</v>
+        <v>36360.61867227482</v>
       </c>
       <c r="D21" s="45" t="inlineStr">
         <is>
@@ -3574,11 +3612,11 @@
           <t>三、投资回报验证（按建议收购价格）</t>
         </is>
       </c>
-      <c r="C23" s="6" t="n"/>
-      <c r="D23" s="6" t="n"/>
-      <c r="E23" s="6" t="n"/>
-      <c r="F23" s="6" t="n"/>
-      <c r="G23" s="6" t="n"/>
+      <c r="C23" s="81" t="n"/>
+      <c r="D23" s="81" t="n"/>
+      <c r="E23" s="81" t="n"/>
+      <c r="F23" s="81" t="n"/>
+      <c r="G23" s="82" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="16" t="inlineStr">
@@ -3607,9 +3645,10 @@
       <c r="C25" s="47" t="n">
         <v>0.12</v>
       </c>
-      <c r="D25" s="16">
-        <f> MARR = 12%</f>
-        <v/>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>MARR = 12%</t>
+        </is>
       </c>
       <c r="E25" s="6" t="n"/>
       <c r="F25" s="6" t="n"/>
@@ -3640,7 +3679,7 @@
         </is>
       </c>
       <c r="C27" s="48" t="n">
-        <v>1.21528630725515</v>
+        <v>1.215005725336249</v>
       </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
@@ -3720,11 +3759,11 @@
           <t>Step 3：敏感性分析 – 建议收购对价（万元，MARR=12%）</t>
         </is>
       </c>
-      <c r="C1" s="6" t="n"/>
-      <c r="D1" s="6" t="n"/>
-      <c r="E1" s="6" t="n"/>
-      <c r="F1" s="6" t="n"/>
-      <c r="G1" s="6" t="n"/>
+      <c r="C1" s="81" t="n"/>
+      <c r="D1" s="81" t="n"/>
+      <c r="E1" s="81" t="n"/>
+      <c r="F1" s="81" t="n"/>
+      <c r="G1" s="82" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="18" t="inlineStr">
@@ -3732,11 +3771,11 @@
           <t>分析变量：稳定期（2027-2029年）出租率 × 2029年租金增长率；底色越深代表收购价格越高。</t>
         </is>
       </c>
-      <c r="C2" s="6" t="n"/>
-      <c r="D2" s="6" t="n"/>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="6" t="n"/>
-      <c r="G2" s="6" t="n"/>
+      <c r="C2" s="81" t="n"/>
+      <c r="D2" s="81" t="n"/>
+      <c r="E2" s="81" t="n"/>
+      <c r="F2" s="81" t="n"/>
+      <c r="G2" s="82" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="6" t="n"/>
@@ -3785,19 +3824,19 @@
         </is>
       </c>
       <c r="C5" s="50" t="n">
-        <v>19953.99989712089</v>
+        <v>19413.38036826641</v>
       </c>
       <c r="D5" s="51" t="n">
-        <v>20682.81821109013</v>
+        <v>20142.19868223565</v>
       </c>
       <c r="E5" s="52" t="n">
-        <v>21411.63652505938</v>
+        <v>20871.01699620491</v>
       </c>
       <c r="F5" s="53" t="n">
-        <v>21897.51540103888</v>
+        <v>21356.8958721844</v>
       </c>
       <c r="G5" s="54" t="n">
-        <v>22626.33371500814</v>
+        <v>22085.71418615365</v>
       </c>
     </row>
     <row r="6">
@@ -3807,19 +3846,19 @@
         </is>
       </c>
       <c r="C6" s="55" t="n">
-        <v>22218.47293940942</v>
+        <v>21787.60738203464</v>
       </c>
       <c r="D6" s="56" t="n">
-        <v>22999.34970437648</v>
+        <v>22568.48414700169</v>
       </c>
       <c r="E6" s="57" t="n">
-        <v>23780.22646934352</v>
+        <v>23349.36091196874</v>
       </c>
       <c r="F6" s="58" t="n">
-        <v>24300.81097932156</v>
+        <v>23869.94542194678</v>
       </c>
       <c r="G6" s="59" t="n">
-        <v>25081.68774428861</v>
+        <v>24650.82218691383</v>
       </c>
     </row>
     <row r="7">
@@ -3829,19 +3868,19 @@
         </is>
       </c>
       <c r="C7" s="60" t="n">
-        <v>24482.94598169797</v>
+        <v>24161.83439580287</v>
       </c>
       <c r="D7" s="61" t="n">
-        <v>25315.88119766283</v>
+        <v>24994.76961176773</v>
       </c>
       <c r="E7" s="62" t="n">
-        <v>26148.81641362769</v>
+        <v>25827.70482773258</v>
       </c>
       <c r="F7" s="63" t="n">
-        <v>26704.10655760425</v>
+        <v>26382.99497170916</v>
       </c>
       <c r="G7" s="64" t="n">
-        <v>27537.04177356911</v>
+        <v>27215.93018767402</v>
       </c>
     </row>
     <row r="8">
@@ -3851,19 +3890,19 @@
         </is>
       </c>
       <c r="C8" s="65" t="n">
-        <v>26747.4190239865</v>
+        <v>26536.0614095711</v>
       </c>
       <c r="D8" s="66" t="n">
-        <v>27632.41269094916</v>
+        <v>27421.05507653376</v>
       </c>
       <c r="E8" s="67" t="n">
-        <v>28517.40635791183</v>
+        <v>28306.04874349642</v>
       </c>
       <c r="F8" s="68" t="n">
-        <v>29107.40213588694</v>
+        <v>28896.04452147153</v>
       </c>
       <c r="G8" s="69" t="n">
-        <v>29992.3958028496</v>
+        <v>29781.03818843418</v>
       </c>
     </row>
     <row r="9">
@@ -3873,19 +3912,19 @@
         </is>
       </c>
       <c r="C9" s="70" t="n">
-        <v>29011.89206627505</v>
+        <v>28910.28842333934</v>
       </c>
       <c r="D9" s="71" t="n">
-        <v>29948.94418423551</v>
+        <v>29847.3405412998</v>
       </c>
       <c r="E9" s="72" t="n">
-        <v>30885.99630219598</v>
+        <v>30784.39265926027</v>
       </c>
       <c r="F9" s="73" t="n">
-        <v>31510.69771416961</v>
+        <v>31409.0940712339</v>
       </c>
       <c r="G9" s="74" t="n">
-        <v>32447.74983213009</v>
+        <v>32346.14618919438</v>
       </c>
     </row>
     <row r="10">
@@ -3895,19 +3934,19 @@
         </is>
       </c>
       <c r="C10" s="75" t="n">
-        <v>31276.36510856359</v>
+        <v>31284.51543710757</v>
       </c>
       <c r="D10" s="76" t="n">
-        <v>32265.47567752186</v>
+        <v>32273.62600606584</v>
       </c>
       <c r="E10" s="31" t="n">
-        <v>33254.58624648013</v>
+        <v>33262.73657502409</v>
       </c>
       <c r="F10" s="77" t="n">
-        <v>33913.9932924523</v>
+        <v>33922.14362099628</v>
       </c>
       <c r="G10" s="78" t="n">
-        <v>34903.10386141056</v>
+        <v>34911.25418995454</v>
       </c>
     </row>
     <row r="11">
@@ -3924,11 +3963,11 @@
           <t>单变量分析①：出租率变化对收购价格的影响（租金增长率固定3%）</t>
         </is>
       </c>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
-      <c r="E12" s="6" t="n"/>
-      <c r="F12" s="6" t="n"/>
-      <c r="G12" s="6" t="n"/>
+      <c r="C12" s="81" t="n"/>
+      <c r="D12" s="81" t="n"/>
+      <c r="E12" s="81" t="n"/>
+      <c r="F12" s="81" t="n"/>
+      <c r="G12" s="82" t="n"/>
     </row>
     <row r="13">
       <c r="B13" s="8" t="inlineStr">
@@ -3957,10 +3996,10 @@
         </is>
       </c>
       <c r="C14" s="21" t="n">
-        <v>21411.63652505938</v>
+        <v>20871.01699620491</v>
       </c>
       <c r="D14" s="79" t="n">
-        <v>-0.3561298172120327</v>
+        <v>-0.3725405921088202</v>
       </c>
       <c r="E14" s="6" t="n"/>
       <c r="F14" s="6" t="n"/>
@@ -3973,10 +4012,10 @@
         </is>
       </c>
       <c r="C15" s="21" t="n">
-        <v>23780.22646934352</v>
+        <v>23349.36091196874</v>
       </c>
       <c r="D15" s="79" t="n">
-        <v>-0.2849038537696265</v>
+        <v>-0.2980324736870562</v>
       </c>
       <c r="E15" s="6" t="n"/>
       <c r="F15" s="6" t="n"/>
@@ -3989,10 +4028,10 @@
         </is>
       </c>
       <c r="C16" s="21" t="n">
-        <v>26148.81641362769</v>
+        <v>25827.70482773258</v>
       </c>
       <c r="D16" s="79" t="n">
-        <v>-0.2136778903272194</v>
+        <v>-0.2235243552652921</v>
       </c>
       <c r="E16" s="6" t="n"/>
       <c r="F16" s="6" t="n"/>
@@ -4005,10 +4044,10 @@
         </is>
       </c>
       <c r="C17" s="21" t="n">
-        <v>28517.40635791183</v>
+        <v>28306.04874349642</v>
       </c>
       <c r="D17" s="79" t="n">
-        <v>-0.1424519268848133</v>
+        <v>-0.1490162368435279</v>
       </c>
       <c r="E17" s="6" t="n"/>
       <c r="F17" s="6" t="n"/>
@@ -4021,10 +4060,10 @@
         </is>
       </c>
       <c r="C18" s="21" t="n">
-        <v>30885.99630219598</v>
+        <v>30784.39265926027</v>
       </c>
       <c r="D18" s="79" t="n">
-        <v>-0.07122596344240666</v>
+        <v>-0.07450811842176375</v>
       </c>
       <c r="E18" s="6" t="n"/>
       <c r="F18" s="6" t="n"/>
@@ -4037,7 +4076,7 @@
         </is>
       </c>
       <c r="C19" s="29" t="n">
-        <v>33254.58624648013</v>
+        <v>33262.73657502409</v>
       </c>
       <c r="D19" s="80" t="n">
         <v>0</v>
@@ -4060,11 +4099,11 @@
           <t>单变量分析②：2029年租金增长率变化对收购价格的影响（出租率固定95%）</t>
         </is>
       </c>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
+      <c r="C21" s="81" t="n"/>
+      <c r="D21" s="81" t="n"/>
+      <c r="E21" s="81" t="n"/>
+      <c r="F21" s="81" t="n"/>
+      <c r="G21" s="82" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="8" t="inlineStr">
@@ -4093,10 +4132,10 @@
         </is>
       </c>
       <c r="C23" s="21" t="n">
-        <v>31276.36510856359</v>
+        <v>31284.51543710757</v>
       </c>
       <c r="D23" s="79" t="n">
-        <v>-0.05948716737156602</v>
+        <v>-0.05947259130212112</v>
       </c>
       <c r="E23" s="6" t="n"/>
       <c r="F23" s="6" t="n"/>
@@ -4109,10 +4148,10 @@
         </is>
       </c>
       <c r="C24" s="21" t="n">
-        <v>32265.47567752186</v>
+        <v>32273.62600606584</v>
       </c>
       <c r="D24" s="79" t="n">
-        <v>-0.02974358368578319</v>
+        <v>-0.0297362956510604</v>
       </c>
       <c r="E24" s="6" t="n"/>
       <c r="F24" s="6" t="n"/>
@@ -4125,7 +4164,7 @@
         </is>
       </c>
       <c r="C25" s="29" t="n">
-        <v>33254.58624648013</v>
+        <v>33262.73657502409</v>
       </c>
       <c r="D25" s="80" t="n">
         <v>0</v>
@@ -4141,10 +4180,10 @@
         </is>
       </c>
       <c r="C26" s="21" t="n">
-        <v>33913.9932924523</v>
+        <v>33922.14362099628</v>
       </c>
       <c r="D26" s="80" t="n">
-        <v>0.01982905579052165</v>
+        <v>0.01982419710070737</v>
       </c>
       <c r="E26" s="6" t="n"/>
       <c r="F26" s="6" t="n"/>
@@ -4157,10 +4196,10 @@
         </is>
       </c>
       <c r="C27" s="21" t="n">
-        <v>34903.10386141056</v>
+        <v>34911.25418995454</v>
       </c>
       <c r="D27" s="80" t="n">
-        <v>0.0495726394763043</v>
+        <v>0.04956049275176788</v>
       </c>
       <c r="E27" s="6" t="n"/>
       <c r="F27" s="6" t="n"/>
@@ -4188,16 +4227,16 @@
           <t>敏感性结论</t>
         </is>
       </c>
-      <c r="C30" s="6" t="n"/>
-      <c r="D30" s="6" t="n"/>
-      <c r="E30" s="6" t="n"/>
-      <c r="F30" s="6" t="n"/>
-      <c r="G30" s="6" t="n"/>
+      <c r="C30" s="81" t="n"/>
+      <c r="D30" s="81" t="n"/>
+      <c r="E30" s="81" t="n"/>
+      <c r="F30" s="81" t="n"/>
+      <c r="G30" s="82" t="n"/>
     </row>
     <row r="31" ht="48" customHeight="1">
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t>基准假设（出租率95%，租金增长率3%）下建议收购价约 33255 万元（3.33亿元）。出租率每下降5%，收购对价降低约2369万元；若出租率仅达80%（最悲观），合理价格约25316万元。</t>
+          <t>基准假设（出租率95%，租金增长率3%）下建议收购价约 33263 万元（3.33亿元）。按“2026年出租率=稳定期出租率-15个百分点”的口径，出租率每下降5个百分点，收购对价约下降2478万元；若稳定出租率仅70%且2029年租金增长率为-3%，合理价格约19413万元。</t>
         </is>
       </c>
       <c r="C31" s="6" t="n"/>

</xml_diff>

<commit_message>
Polish final report and workbook
</commit_message>
<xml_diff>
--- a/final_report/宁波怡丰汇投资分析.xlsx
+++ b/final_report/宁波怡丰汇投资分析.xlsx
@@ -26,7 +26,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="21">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -115,8 +115,37 @@
       <color rgb="00375623"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="001F3A5F"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="39">
+  <fills count="42">
     <fill>
       <patternFill/>
     </fill>
@@ -308,8 +337,23 @@
         <fgColor rgb="00C80080"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F81BD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCE6F1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -375,11 +419,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="111">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -617,6 +724,76 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="39" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="40" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="18" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="41" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="18" fillId="41" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -3161,8 +3338,8 @@
       <c r="E19" s="81" t="n"/>
       <c r="F19" s="82" t="n"/>
     </row>
-    <row r="20">
-      <c r="B20" s="41" t="inlineStr">
+    <row r="20" ht="30" customHeight="1">
+      <c r="B20" s="101" t="inlineStr">
         <is>
           <t>Q1 → Q2：运营启动（仅停车费+物业费），税前利润由0→负（因分摊的人事/管理/能耗成本较高）</t>
         </is>
@@ -3172,8 +3349,8 @@
       <c r="E20" s="6" t="n"/>
       <c r="F20" s="6" t="n"/>
     </row>
-    <row r="21">
-      <c r="B21" s="41" t="inlineStr">
+    <row r="21" ht="30" customHeight="1">
+      <c r="B21" s="101" t="inlineStr">
         <is>
           <t>Q2 → Q3：免租期结束，租金收入开始确认，季度税前利润大幅转正（约+1150万元）</t>
         </is>
@@ -3183,8 +3360,8 @@
       <c r="E21" s="6" t="n"/>
       <c r="F21" s="6" t="n"/>
     </row>
-    <row r="22">
-      <c r="B22" s="41" t="inlineStr">
+    <row r="22" ht="24" customHeight="1">
+      <c r="B22" s="101" t="inlineStr">
         <is>
           <t>Q3 = Q4（2026）：同等运营条件，现金流基本持平</t>
         </is>
@@ -3194,8 +3371,8 @@
       <c r="E22" s="6" t="n"/>
       <c r="F22" s="6" t="n"/>
     </row>
-    <row r="23">
-      <c r="B23" s="42" t="inlineStr">
+    <row r="23" ht="38" customHeight="1">
+      <c r="B23" s="102" t="inlineStr">
         <is>
           <t>改造期年度净CF（2026）≈ 1103万元  vs  稳定期（2027）≈ 3325万元，相差约2222万元（约202%增幅）</t>
         </is>
@@ -3213,14 +3390,18 @@
       <c r="F24" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="11">
+    <mergeCell ref="B21:F21"/>
     <mergeCell ref="B12:F12"/>
     <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B20:F20"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B1:F1"/>
+    <mergeCell ref="B22:F22"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3236,12 +3417,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3277,126 +3458,134 @@
       <c r="G3" s="82" t="n"/>
     </row>
     <row r="4">
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="90" t="inlineStr">
         <is>
           <t>时间节点</t>
         </is>
       </c>
-      <c r="C4" s="8" t="inlineStr">
+      <c r="C4" s="90" t="inlineStr">
         <is>
           <t>期间</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr">
+      <c r="D4" s="90" t="inlineStr">
         <is>
           <t>年度总CF（万元）</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="90" t="inlineStr">
         <is>
           <t>折现系数</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="90" t="inlineStr">
         <is>
           <t>现值（万元）</t>
         </is>
       </c>
-      <c r="G4" s="6" t="n"/>
-    </row>
-    <row r="5">
-      <c r="B5" s="9" t="inlineStr">
+      <c r="G4" s="91" t="n"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="92" t="inlineStr">
         <is>
           <t>2026年</t>
         </is>
       </c>
-      <c r="C5" s="16" t="n">
+      <c r="C5" s="93" t="inlineStr">
+        <is>
+          <t>改造期（9个月运营）</t>
+        </is>
+      </c>
+      <c r="D5" s="21" t="n">
         <v>1102.6621010475</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="E5" s="43" t="n">
         <v>0.8928571428571428</v>
       </c>
-      <c r="E5" s="43" t="n">
+      <c r="F5" s="94" t="n">
         <v>984.5197330781251</v>
       </c>
-      <c r="F5" s="29" t="n">
-        <v>984.5197330781253</v>
-      </c>
-      <c r="G5" s="6" t="n"/>
-    </row>
-    <row r="6">
-      <c r="B6" s="9" t="inlineStr">
+      <c r="G5" s="95" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="92" t="inlineStr">
         <is>
           <t>2027年</t>
         </is>
       </c>
-      <c r="C6" s="16" t="n">
+      <c r="C6" s="93" t="inlineStr">
+        <is>
+          <t>稳定期</t>
+        </is>
+      </c>
+      <c r="D6" s="21" t="n">
         <v>3324.527119720312</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="E6" s="43" t="n">
         <v>0.7971938775510203</v>
       </c>
-      <c r="E6" s="43" t="n">
+      <c r="F6" s="94" t="n">
         <v>2650.292665593361</v>
       </c>
-      <c r="F6" s="29" t="n">
-        <v>2650.292665593362</v>
-      </c>
-      <c r="G6" s="6" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="9" t="inlineStr">
+      <c r="G6" s="95" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="92" t="inlineStr">
         <is>
           <t>2028年</t>
         </is>
       </c>
-      <c r="C7" s="16" t="n">
+      <c r="C7" s="93" t="inlineStr">
+        <is>
+          <t>稳定期</t>
+        </is>
+      </c>
+      <c r="D7" s="21" t="n">
         <v>3376.8402593355</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="E7" s="43" t="n">
         <v>0.7117802478134109</v>
       </c>
-      <c r="E7" s="43" t="n">
+      <c r="F7" s="94" t="n">
         <v>2403.568196616125</v>
       </c>
-      <c r="F7" s="29" t="n">
-        <v>2395.173358215821</v>
-      </c>
-      <c r="G7" s="6" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="9" t="inlineStr">
+      <c r="G7" s="95" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="92" t="inlineStr">
         <is>
           <t>2029年</t>
         </is>
       </c>
-      <c r="C8" s="16" t="n">
+      <c r="C8" s="93" t="inlineStr">
+        <is>
+          <t>稳定期 + 退出价值</t>
+        </is>
+      </c>
+      <c r="D8" s="21" t="n">
         <v>47712.62865266857</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="E8" s="43" t="n">
         <v>0.6355180784048311</v>
       </c>
-      <c r="E8" s="43" t="n">
+      <c r="F8" s="94" t="n">
         <v>30322.23807698721</v>
       </c>
-      <c r="F8" s="29" t="n">
-        <v>30322.23807698723</v>
-      </c>
-      <c r="G8" s="6" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="20" t="inlineStr">
+      <c r="G8" s="95" t="n"/>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="96" t="inlineStr">
         <is>
           <t>未来CF现值合计</t>
         </is>
       </c>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="44" t="n">
+      <c r="C9" s="97" t="n"/>
+      <c r="D9" s="98" t="n"/>
+      <c r="E9" s="99" t="n"/>
+      <c r="F9" s="100" t="n">
         <v>36360.61867227482</v>
       </c>
-      <c r="G9" s="6" t="n"/>
+      <c r="G9" s="95" t="n"/>
     </row>
     <row r="10">
       <c r="B10" s="6" t="n"/>
@@ -3472,7 +3661,7 @@
       <c r="F14" s="6" t="n"/>
       <c r="G14" s="6" t="n"/>
     </row>
-    <row r="15">
+    <row r="15" ht="34" customHeight="1">
       <c r="B15" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">  = 可用于支付收购对价×(1+3%)</t>
@@ -3515,7 +3704,7 @@
         </is>
       </c>
       <c r="C17" s="31" t="n">
-        <v>33262.73657502409</v>
+        <v>33262.7365750241</v>
       </c>
       <c r="D17" s="45" t="inlineStr">
         <is>
@@ -3533,7 +3722,7 @@
         </is>
       </c>
       <c r="C18" s="21" t="n">
-        <v>997.8820972507227</v>
+        <v>997.8820972507229</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
@@ -3580,7 +3769,7 @@
       <c r="F20" s="6" t="n"/>
       <c r="G20" s="6" t="n"/>
     </row>
-    <row r="21">
+    <row r="21" ht="34" customHeight="1">
       <c r="B21" s="30" t="inlineStr">
         <is>
           <t>★ 总投资额（P×1.03 + 2100万）</t>
@@ -3741,7 +3930,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G32"/>
+  <dimension ref="B1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -4233,31 +4422,36 @@
       <c r="F30" s="81" t="n"/>
       <c r="G30" s="82" t="n"/>
     </row>
-    <row r="31" ht="48" customHeight="1">
-      <c r="B31" s="16" t="inlineStr">
+    <row r="31" ht="34" customHeight="1">
+      <c r="B31" s="103" t="inlineStr">
         <is>
           <t>基准假设（出租率95%，租金增长率3%）下建议收购价约 33263 万元（3.33亿元）。按“2026年出租率=稳定期出租率-15个百分点”的口径，出租率每下降5个百分点，收购对价约下降2478万元；若稳定出租率仅70%且2029年租金增长率为-3%，合理价格约19413万元。</t>
         </is>
       </c>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
-    </row>
-    <row r="32">
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
+      <c r="C31" s="104" t="n"/>
+      <c r="D31" s="104" t="n"/>
+      <c r="E31" s="104" t="n"/>
+      <c r="F31" s="104" t="n"/>
+      <c r="G31" s="105" t="n"/>
+    </row>
+    <row r="32" ht="34" customHeight="1">
+      <c r="B32" s="106" t="n"/>
+      <c r="G32" s="107" t="n"/>
+    </row>
+    <row r="33" ht="28" customHeight="1">
+      <c r="B33" s="108" t="n"/>
+      <c r="C33" s="109" t="n"/>
+      <c r="D33" s="109" t="n"/>
+      <c r="E33" s="109" t="n"/>
+      <c r="F33" s="109" t="n"/>
+      <c r="G33" s="110" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="6">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B30:G30"/>
     <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B31:G33"/>
     <mergeCell ref="B12:G12"/>
     <mergeCell ref="B21:G21"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fix workbook preview formulas
</commit_message>
<xml_diff>
--- a/final_report/宁波怡丰汇投资分析.xlsx
+++ b/final_report/宁波怡丰汇投资分析.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\课程文件\工程经济学\case_study\EngineringEconomyCaseStudy\final_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9734FF0-A83E-4762-A535-EFB76F4A6DDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{015D3657-E860-41C0-83E9-CC0C2F3A160E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="11332" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,14 +19,22 @@
     <sheet name="季度现金流" sheetId="4" r:id="rId4"/>
     <sheet name="收购价格" sheetId="5" r:id="rId5"/>
     <sheet name="敏感性分析" sheetId="6" r:id="rId6"/>
-    <sheet name="敏感性计算明细" sheetId="7" r:id="rId7"/>
+    <sheet name="敏感性计算明细" sheetId="7" state="hidden" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">封面!$B$1:$F$14</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">季度现金流!$B$1:$G$24</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">敏感性分析!$B$1:$G$32</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">年度现金流!$B$1:$G$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">收购价格!$B$1:$F$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">主要假设!$B$1:$G$65</definedName>
+  </definedNames>
   <calcPr calcId="191029" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="259">
   <si>
     <t>宁波怡丰汇商业项目</t>
   </si>
@@ -594,6 +602,9 @@
   </si>
   <si>
     <t>敏感性结论</t>
+  </si>
+  <si>
+    <t>基准假设（出租率95%，租金增长率3%）下建议收购价约 33263 万元（3.33亿元）。按“2026年出租率=稳定期出租率-15个百分点”的口径，出租率每下降5个百分点，收购对价约下降2478万元；若稳定出租率仅70%且2029年租金增长率为-3%，合理价格约19413万元。</t>
   </si>
   <si>
     <t>敏感性计算明细：稳定期出租率 × 2029年租金增长率</t>
@@ -815,7 +826,7 @@
     <numFmt numFmtId="177" formatCode="0.0%"/>
     <numFmt numFmtId="178" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -976,6 +987,13 @@
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Microsoft YaHei"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Microsoft YaHei"/>
       <family val="2"/>
       <charset val="134"/>
@@ -1585,42 +1603,42 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -1933,6 +1951,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:B13"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
@@ -1995,12 +2016,16 @@
     <mergeCell ref="B2:B3"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:H65"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
@@ -3022,12 +3047,16 @@
     <mergeCell ref="B3:H3"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
+  <pageSetup paperSize="9" scale="93" fitToHeight="0" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:G34"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
@@ -3099,19 +3128,19 @@
         <v>87</v>
       </c>
       <c r="C6" s="14">
-        <f>SUMPRODUCT(主要假设!$E$5:$E$12,主要假设!$C$16:$C$23)*主要假设!C27*主要假设!E27*(1+主要假设!D27)/10000</f>
+        <f>156104.99*0.8*184*(1+0)/10000</f>
         <v>2297.8654528000002</v>
       </c>
       <c r="D6" s="14">
-        <f>SUMPRODUCT(主要假设!$E$5:$E$12,主要假设!$C$16:$C$23)*主要假设!C28*主要假设!E28*(1+主要假设!D28)/10000</f>
+        <f>156104.99*0.95*365*(1+0)/10000</f>
         <v>5412.9405282499993</v>
       </c>
       <c r="E6" s="14">
-        <f>SUMPRODUCT(主要假设!$E$5:$E$12,主要假设!$C$16:$C$23)*主要假设!C29*主要假设!E29*(1+主要假设!D29)/10000</f>
+        <f>156104.99*0.95*366*(1+0)/10000</f>
         <v>5427.7705022999999</v>
       </c>
       <c r="F6" s="14">
-        <f>SUMPRODUCT(主要假设!$E$5:$E$12,主要假设!$C$16:$C$23)*主要假设!C30*主要假设!E30*(1+主要假设!D30)/10000</f>
+        <f>156104.99*0.95*365*(1+0.03)/10000</f>
         <v>5575.3287440974991</v>
       </c>
       <c r="G6" s="3"/>
@@ -3121,19 +3150,19 @@
         <v>88</v>
       </c>
       <c r="C7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!C34*主要假设!D34*主要假设!E34*主要假设!F27/10000</f>
+        <f>1005*3*6*0.5*275/10000</f>
         <v>248.73750000000001</v>
       </c>
       <c r="D7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!C35*主要假设!D35*主要假设!E35*主要假设!F28/10000</f>
+        <f>1005*3*6*0.6*365/10000</f>
         <v>396.17099999999999</v>
       </c>
       <c r="E7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!C36*主要假设!D36*主要假设!E36*主要假设!F29/10000</f>
+        <f>1005*3*6*0.7*366/10000</f>
         <v>463.4658</v>
       </c>
       <c r="F7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!C37*主要假设!D37*主要假设!E37*主要假设!F30/10000</f>
+        <f>1005*3*6*0.8*365/10000</f>
         <v>528.22799999999995</v>
       </c>
       <c r="G7" s="3"/>
@@ -3143,19 +3172,19 @@
         <v>89</v>
       </c>
       <c r="C8" s="14">
-        <f>主要假设!$E$13*主要假设!C27*10*(12-主要假设!$C$64)/10000</f>
+        <f>62629.76*0.8*10*9/10000</f>
         <v>450.93427200000008</v>
       </c>
       <c r="D8" s="14">
-        <f>主要假设!$E$13*主要假设!C28*10*12/10000</f>
+        <f>62629.76*0.95*10*12/10000</f>
         <v>713.97926399999994</v>
       </c>
       <c r="E8" s="14">
-        <f>主要假设!$E$13*主要假设!C29*10*12/10000</f>
+        <f>62629.76*0.95*10*12/10000</f>
         <v>713.97926399999994</v>
       </c>
       <c r="F8" s="14">
-        <f>主要假设!$E$13*主要假设!C30*10*12/10000</f>
+        <f>62629.76*0.95*10*12/10000</f>
         <v>713.97926399999994</v>
       </c>
       <c r="G8" s="3"/>
@@ -3165,19 +3194,19 @@
         <v>90</v>
       </c>
       <c r="C9" s="16">
-        <f>SUM(C6:C8)</f>
+        <f>C6+C7+C8</f>
         <v>2997.5372248000003</v>
       </c>
       <c r="D9" s="16">
-        <f>SUM(D6:D8)</f>
+        <f>D6+D7+D8</f>
         <v>6523.0907922499991</v>
       </c>
       <c r="E9" s="16">
-        <f>SUM(E6:E8)</f>
+        <f>E6+E7+E8</f>
         <v>6605.2155662999994</v>
       </c>
       <c r="F9" s="16">
-        <f>SUM(F6:F8)</f>
+        <f>F6+F7+F8</f>
         <v>6817.5360080974988</v>
       </c>
       <c r="G9" s="3"/>
@@ -3197,19 +3226,19 @@
         <v>92</v>
       </c>
       <c r="C11" s="14">
-        <f>主要假设!$C$40/10000*(12-主要假设!$C$64)/12</f>
+        <f>5000000/10000*9/12</f>
         <v>375</v>
       </c>
       <c r="D11" s="14">
-        <f>主要假设!$C$40/10000*(1+主要假设!D50)</f>
+        <f>5000000/10000</f>
         <v>500</v>
       </c>
       <c r="E11" s="14">
-        <f>D11*(1+主要假设!E50)</f>
+        <f>D11*(1+3%)</f>
         <v>515</v>
       </c>
       <c r="F11" s="14">
-        <f>E11*(1+主要假设!F50)</f>
+        <f>E11</f>
         <v>515</v>
       </c>
       <c r="G11" s="3"/>
@@ -3219,19 +3248,19 @@
         <v>93</v>
       </c>
       <c r="C12" s="14">
-        <f>主要假设!$C$41/10000*(12-主要假设!$C$64)/12</f>
+        <f>5000000/10000*9/12</f>
         <v>375</v>
       </c>
       <c r="D12" s="14">
-        <f>主要假设!$C$41/10000*(1+主要假设!D51)</f>
+        <f>5000000/10000*(1-5%)</f>
         <v>475</v>
       </c>
       <c r="E12" s="14">
-        <f>D12*(1+主要假设!E51)</f>
+        <f>D12*(1-5%)</f>
         <v>451.25</v>
       </c>
       <c r="F12" s="14">
-        <f>E12*(1+主要假设!F51)</f>
+        <f>E12*(1-5%)</f>
         <v>428.6875</v>
       </c>
       <c r="G12" s="3"/>
@@ -3241,19 +3270,19 @@
         <v>94</v>
       </c>
       <c r="C13" s="14">
-        <f>主要假设!$C$13*主要假设!$C$42/10000*(12-主要假设!$C$64)/12</f>
+        <f>107039.13*15/10000*9/12</f>
         <v>120.41902125000001</v>
       </c>
       <c r="D13" s="14">
-        <f>主要假设!$C$13*主要假设!$C$42/10000*(1+主要假设!D52)</f>
+        <f>107039.13*15/10000*(1+3%)</f>
         <v>165.37545585000004</v>
       </c>
       <c r="E13" s="14">
-        <f>D13*(1+主要假设!E52)</f>
+        <f>D13*(1+3%)</f>
         <v>170.33671952550003</v>
       </c>
       <c r="F13" s="14">
-        <f>E13*(1+主要假设!F52)</f>
+        <f>E13*(1+3%)</f>
         <v>175.44682111126502</v>
       </c>
       <c r="G13" s="3"/>
@@ -3263,19 +3292,19 @@
         <v>95</v>
       </c>
       <c r="C14" s="14">
-        <f>C6*主要假设!$C$43</f>
+        <f>C6*2.5%</f>
         <v>57.44663632000001</v>
       </c>
       <c r="D14" s="14">
-        <f>D6*主要假设!$C$43</f>
+        <f>D6*2.5%</f>
         <v>135.32351320625</v>
       </c>
       <c r="E14" s="14">
-        <f>E6*主要假设!$C$43</f>
+        <f>E6*2.5%</f>
         <v>135.6942625575</v>
       </c>
       <c r="F14" s="14">
-        <f>F6*主要假设!$C$43</f>
+        <f>F6*2.5%</f>
         <v>139.38321860243749</v>
       </c>
       <c r="G14" s="3"/>
@@ -3285,19 +3314,19 @@
         <v>96</v>
       </c>
       <c r="C15" s="14">
-        <f>主要假设!$C$13*主要假设!$C$44/10000*(12-主要假设!$C$64)/12</f>
+        <f>107039.13*30/10000*9/12</f>
         <v>240.83804250000003</v>
       </c>
       <c r="D15" s="14">
-        <f>主要假设!$C$13*主要假设!$C$44/10000*(1+主要假设!D53)</f>
+        <f>107039.13*30/10000*(1+3%)</f>
         <v>330.75091170000007</v>
       </c>
       <c r="E15" s="14">
-        <f>D15*(1+主要假设!E53)</f>
+        <f>D15*(1+3%)</f>
         <v>340.67343905100006</v>
       </c>
       <c r="F15" s="14">
-        <f>E15*(1+主要假设!F53)</f>
+        <f>E15*(1+3%)</f>
         <v>350.89364222253005</v>
       </c>
       <c r="G15" s="3"/>
@@ -3307,19 +3336,19 @@
         <v>97</v>
       </c>
       <c r="C16" s="14">
-        <f>主要假设!$C$13*主要假设!$C$45/10000*(12-主要假设!$C$64)/12</f>
+        <f>107039.13*40/10000*9/12</f>
         <v>321.11739</v>
       </c>
       <c r="D16" s="14">
-        <f>主要假设!$C$13*主要假设!$C$45/10000*(1+主要假设!D54)</f>
+        <f>107039.13*40/10000*(1+1%)</f>
         <v>432.43808519999999</v>
       </c>
       <c r="E16" s="14">
-        <f>D16*(1+主要假设!E54)</f>
+        <f>D16*(1+1%)</f>
         <v>436.76246605199998</v>
       </c>
       <c r="F16" s="14">
-        <f>E16*(1+主要假设!F54)</f>
+        <f>E16*(1+1%)</f>
         <v>441.13009071251997</v>
       </c>
       <c r="G16" s="3"/>
@@ -3329,19 +3358,19 @@
         <v>98</v>
       </c>
       <c r="C17" s="14">
-        <f>主要假设!$C$46/10000*(12-主要假设!$C$64)/12</f>
+        <f>500000/10000*9/12</f>
         <v>37.5</v>
       </c>
       <c r="D17" s="14">
-        <f>主要假设!$C$46/10000*(1+主要假设!D55)</f>
+        <f>500000/10000*(1+3%)</f>
         <v>51.5</v>
       </c>
       <c r="E17" s="14">
-        <f>D17*(1+主要假设!E55)</f>
+        <f>D17*(1+3%)</f>
         <v>53.045000000000002</v>
       </c>
       <c r="F17" s="14">
-        <f>E17*(1+主要假设!F55)</f>
+        <f>E17*(1+3%)</f>
         <v>54.63635</v>
       </c>
       <c r="G17" s="3"/>
@@ -3351,19 +3380,19 @@
         <v>99</v>
       </c>
       <c r="C18" s="18">
-        <f>SUM(C11:C17)</f>
+        <f>C11+C12+C13+C14+C15+C16+C17</f>
         <v>1527.3210900700001</v>
       </c>
       <c r="D18" s="18">
-        <f>SUM(D11:D17)</f>
+        <f>D11+D12+D13+D14+D15+D16+D17</f>
         <v>2090.3879659562499</v>
       </c>
       <c r="E18" s="18">
-        <f>SUM(E11:E17)</f>
+        <f>E11+E12+E13+E14+E15+E16+E17</f>
         <v>2102.761887186</v>
       </c>
       <c r="F18" s="18">
-        <f>SUM(F11:F17)</f>
+        <f>F11+F12+F13+F14+F15+F16+F17</f>
         <v>2105.1776226487527</v>
       </c>
       <c r="G18" s="3"/>
@@ -3405,19 +3434,19 @@
         <v>102</v>
       </c>
       <c r="C21" s="14">
-        <f>MAX(C20,0)*主要假设!$C$61</f>
+        <f>C20*25%</f>
         <v>367.55403368250006</v>
       </c>
       <c r="D21" s="14">
-        <f>MAX(D20,0)*主要假设!$C$61</f>
+        <f>D20*25%</f>
         <v>1108.1757065734373</v>
       </c>
       <c r="E21" s="14">
-        <f>MAX(E20,0)*主要假设!$C$61</f>
+        <f>E20*25%</f>
         <v>1125.6134197785</v>
       </c>
       <c r="F21" s="14">
-        <f>MAX(F20,0)*主要假设!$C$61</f>
+        <f>F20*25%</f>
         <v>1178.0895963621865</v>
       </c>
       <c r="G21" s="3"/>
@@ -3462,7 +3491,7 @@
       <c r="D24" s="24"/>
       <c r="E24" s="24"/>
       <c r="F24" s="24">
-        <f>F22/主要假设!$C$63</f>
+        <f>F22/8%</f>
         <v>44178.359863581994</v>
       </c>
       <c r="G24" s="3"/>
@@ -3522,19 +3551,15 @@
         <v>37</v>
       </c>
       <c r="C29" s="25">
-        <f>主要假设!C27</f>
         <v>0.8</v>
       </c>
       <c r="D29" s="25">
-        <f>主要假设!C28</f>
         <v>0.95</v>
       </c>
       <c r="E29" s="25">
-        <f>主要假设!C29</f>
         <v>0.95</v>
       </c>
       <c r="F29" s="25">
-        <f>主要假设!C30</f>
         <v>0.95</v>
       </c>
       <c r="G29" s="3"/>
@@ -3544,19 +3569,15 @@
         <v>109</v>
       </c>
       <c r="C30" s="11">
-        <f>主要假设!F27</f>
         <v>275</v>
       </c>
       <c r="D30" s="11">
-        <f>主要假设!F28</f>
         <v>365</v>
       </c>
       <c r="E30" s="11">
-        <f>主要假设!F29</f>
         <v>366</v>
       </c>
       <c r="F30" s="11">
-        <f>主要假设!F30</f>
         <v>365</v>
       </c>
       <c r="G30" s="3"/>
@@ -3633,12 +3654,16 @@
     <mergeCell ref="B23:G23"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:F24"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
@@ -3709,11 +3734,11 @@
         <v>0</v>
       </c>
       <c r="E6" s="27">
-        <f>年度现金流!$C$6/主要假设!$E$27*92</f>
+        <f>156104.99*0.8*92/10000</f>
         <v>1148.9327264000001</v>
       </c>
       <c r="F6" s="27">
-        <f>年度现金流!$C$6/主要假设!$E$27*92</f>
+        <f>156104.99*0.8*92/10000</f>
         <v>1148.9327264000001</v>
       </c>
     </row>
@@ -3722,19 +3747,19 @@
         <v>120</v>
       </c>
       <c r="C7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!$C$34*主要假设!$D$34*主要假设!$E$34*0/10000</f>
+        <f>1005*3*6*0.5*0/10000</f>
         <v>0</v>
       </c>
       <c r="D7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!$C$34*主要假设!$D$34*主要假设!$E$34*91/10000</f>
+        <f>1005*3*6*0.5*91/10000</f>
         <v>82.3095</v>
       </c>
       <c r="E7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!$C$34*主要假设!$D$34*主要假设!$E$34*92/10000</f>
+        <f>1005*3*6*0.5*92/10000</f>
         <v>83.213999999999999</v>
       </c>
       <c r="F7" s="14">
-        <f>(主要假设!$F$13+主要假设!$G$13)*主要假设!$C$34*主要假设!$D$34*主要假设!$E$34*92/10000</f>
+        <f>1005*3*6*0.5*92/10000</f>
         <v>83.213999999999999</v>
       </c>
     </row>
@@ -3746,15 +3771,15 @@
         <v>0</v>
       </c>
       <c r="D8" s="14">
-        <f>年度现金流!$C$8/3</f>
+        <f>62629.76*0.8*10*3/10000</f>
         <v>150.31142400000002</v>
       </c>
       <c r="E8" s="14">
-        <f>年度现金流!$C$8/3</f>
+        <f>62629.76*0.8*10*3/10000</f>
         <v>150.31142400000002</v>
       </c>
       <c r="F8" s="14">
-        <f>年度现金流!$C$8/3</f>
+        <f>62629.76*0.8*10*3/10000</f>
         <v>150.31142400000002</v>
       </c>
     </row>
@@ -3763,19 +3788,19 @@
         <v>122</v>
       </c>
       <c r="C9" s="16">
-        <f>SUM(C6:C8)</f>
+        <f>C6+C7+C8</f>
         <v>0</v>
       </c>
       <c r="D9" s="16">
-        <f>SUM(D6:D8)</f>
+        <f>D6+D7+D8</f>
         <v>232.620924</v>
       </c>
       <c r="E9" s="16">
-        <f>SUM(E6:E8)</f>
+        <f>E6+E7+E8</f>
         <v>1382.4581504</v>
       </c>
       <c r="F9" s="16">
-        <f>SUM(F6:F8)</f>
+        <f>F6+F7+F8</f>
         <v>1382.4581504</v>
       </c>
     </row>
@@ -3793,19 +3818,20 @@
         <v>124</v>
       </c>
       <c r="C11" s="29">
+        <f>0</f>
         <v>0</v>
       </c>
       <c r="D11" s="29">
-        <f>年度现金流!$C$18/3</f>
-        <v>509.10703002333338</v>
+        <f>1527.32203941316/3</f>
+        <v>509.10734647105329</v>
       </c>
       <c r="E11" s="29">
-        <f>年度现金流!$C$18/3</f>
-        <v>509.10703002333338</v>
+        <f>1527.32203941316/3</f>
+        <v>509.10734647105329</v>
       </c>
       <c r="F11" s="29">
-        <f>年度现金流!$C$18/3</f>
-        <v>509.10703002333338</v>
+        <f>1527.32203941316/3</f>
+        <v>509.10734647105329</v>
       </c>
     </row>
     <row r="12" spans="2:6" ht="14.65" customHeight="1">
@@ -3827,15 +3853,15 @@
       </c>
       <c r="D13" s="22">
         <f>D9-D11</f>
-        <v>-276.48610602333338</v>
+        <v>-276.48642247105329</v>
       </c>
       <c r="E13" s="22">
         <f>E9-E11</f>
-        <v>873.35112037666659</v>
+        <v>873.35080392894679</v>
       </c>
       <c r="F13" s="22">
         <f>F9-F11</f>
-        <v>873.35112037666659</v>
+        <v>873.35080392894679</v>
       </c>
     </row>
     <row r="14" spans="2:6">
@@ -3868,7 +3894,7 @@
         <v>129</v>
       </c>
       <c r="F16" s="24">
-        <f>年度现金流!$C$22</f>
+        <f>1102.6621010475</f>
         <v>1102.6621010475001</v>
       </c>
     </row>
@@ -3953,12 +3979,16 @@
     <mergeCell ref="B19:F19"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:G30"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
@@ -4025,11 +4055,11 @@
         <v>143</v>
       </c>
       <c r="D5" s="14">
-        <f>年度现金流!C26</f>
+        <f>1102.6621010475</f>
         <v>1102.6621010475001</v>
       </c>
       <c r="E5" s="31">
-        <f>1/(1+主要假设!$C$62)^1</f>
+        <f>1/(1+12%)^1</f>
         <v>0.89285714285714279</v>
       </c>
       <c r="F5" s="71">
@@ -4046,16 +4076,16 @@
         <v>145</v>
       </c>
       <c r="D6" s="14">
-        <f>年度现金流!D26</f>
-        <v>3324.5271197203119</v>
+        <f>3324.52711972031</f>
+        <v>3324.5271197203101</v>
       </c>
       <c r="E6" s="31">
-        <f>1/(1+主要假设!$C$62)^2</f>
+        <f>1/(1+12%)^2</f>
         <v>0.79719387755102034</v>
       </c>
       <c r="F6" s="71">
         <f>D6*E6</f>
-        <v>2650.2926655933607</v>
+        <v>2650.2926655933593</v>
       </c>
       <c r="G6" s="72"/>
     </row>
@@ -4067,11 +4097,11 @@
         <v>145</v>
       </c>
       <c r="D7" s="14">
-        <f>年度现金流!E26</f>
+        <f>3376.8402593355</f>
         <v>3376.8402593354999</v>
       </c>
       <c r="E7" s="31">
-        <f>1/(1+主要假设!$C$62)^3</f>
+        <f>1/(1+12%)^3</f>
         <v>0.71178024781341087</v>
       </c>
       <c r="F7" s="71">
@@ -4088,16 +4118,16 @@
         <v>148</v>
       </c>
       <c r="D8" s="14">
-        <f>年度现金流!F26</f>
-        <v>47712.628652668551</v>
+        <f>47712.6286526685</f>
+        <v>47712.6286526685</v>
       </c>
       <c r="E8" s="31">
-        <f>1/(1+主要假设!$C$62)^4</f>
+        <f>1/(1+12%)^4</f>
         <v>0.63551807840483121</v>
       </c>
       <c r="F8" s="71">
         <f>D8*E8</f>
-        <v>30322.238076987207</v>
+        <v>30322.238076987174</v>
       </c>
       <c r="G8" s="72"/>
     </row>
@@ -4109,8 +4139,8 @@
       <c r="D9" s="75"/>
       <c r="E9" s="76"/>
       <c r="F9" s="77">
-        <f>SUM(F5:F8)</f>
-        <v>36360.618672274817</v>
+        <f>F5+F6+F7+F8</f>
+        <v>36360.618672274781</v>
       </c>
       <c r="G9" s="72"/>
     </row>
@@ -4138,7 +4168,7 @@
       </c>
       <c r="C12" s="14">
         <f>F9</f>
-        <v>36360.618672274817</v>
+        <v>36360.618672274781</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>151</v>
@@ -4152,7 +4182,7 @@
         <v>152</v>
       </c>
       <c r="C13" s="14">
-        <f>-主要假设!$C$59/10000</f>
+        <f>-1100</f>
         <v>-1100</v>
       </c>
       <c r="D13" s="12" t="s">
@@ -4167,7 +4197,7 @@
         <v>153</v>
       </c>
       <c r="C14" s="14">
-        <f>-主要假设!$C$60/10000</f>
+        <f>-1000</f>
         <v>-1000</v>
       </c>
       <c r="D14" s="12" t="s">
@@ -4182,8 +4212,8 @@
         <v>154</v>
       </c>
       <c r="C15" s="22">
-        <f>SUM(C12:C14)</f>
-        <v>34260.618672274817</v>
+        <f>C12+C13+C14</f>
+        <v>34260.618672274781</v>
       </c>
       <c r="D15" s="32" t="s">
         <v>151</v>
@@ -4197,7 +4227,7 @@
         <v>155</v>
       </c>
       <c r="C16" s="33">
-        <f>1+主要假设!$C$58</f>
+        <f>1+3%</f>
         <v>1.03</v>
       </c>
       <c r="D16" s="12" t="s">
@@ -4213,7 +4243,7 @@
       </c>
       <c r="C17" s="22">
         <f>C15/C16</f>
-        <v>33262.736575024093</v>
+        <v>33262.736575024057</v>
       </c>
       <c r="D17" s="32" t="s">
         <v>151</v>
@@ -4227,8 +4257,8 @@
         <v>158</v>
       </c>
       <c r="C18" s="14">
-        <f>C17*主要假设!$C$58</f>
-        <v>997.88209725072272</v>
+        <f>C17*3%</f>
+        <v>997.8820972507217</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>151</v>
@@ -4242,7 +4272,7 @@
         <v>159</v>
       </c>
       <c r="C19" s="14">
-        <f>主要假设!$C$59/10000</f>
+        <f>1100</f>
         <v>1100</v>
       </c>
       <c r="D19" s="12" t="s">
@@ -4257,7 +4287,7 @@
         <v>160</v>
       </c>
       <c r="C20" s="14">
-        <f>主要假设!$C$60/10000</f>
+        <f>1000</f>
         <v>1000</v>
       </c>
       <c r="D20" s="12" t="s">
@@ -4272,8 +4302,8 @@
         <v>161</v>
       </c>
       <c r="C21" s="22">
-        <f>C17*(1+主要假设!$C$58)+C19+C20</f>
-        <v>36360.618672274817</v>
+        <f>C17*(1+3%)+C19+C20</f>
+        <v>36360.618672274781</v>
       </c>
       <c r="D21" s="32" t="s">
         <v>151</v>
@@ -4320,7 +4350,7 @@
         <v>164</v>
       </c>
       <c r="C25" s="34">
-        <f>主要假设!$C$62</f>
+        <f>12%</f>
         <v>0.12</v>
       </c>
       <c r="D25" s="12" t="s">
@@ -4350,8 +4380,8 @@
         <v>167</v>
       </c>
       <c r="C27" s="35">
-        <f>年度现金流!F24/C21</f>
-        <v>1.2150057253362483</v>
+        <f>44178.359863582/C21</f>
+        <v>1.2150057253362496</v>
       </c>
       <c r="D27" s="12" t="s">
         <v>168</v>
@@ -4399,12 +4429,16 @@
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:G33"/>
   <sheetFormatPr defaultRowHeight="13.5"/>
   <cols>
@@ -4466,24 +4500,24 @@
         <v>0.7</v>
       </c>
       <c r="C5" s="36">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B5,敏感性计算明细!$C:$C,C4)</f>
-        <v>19413.380368266404</v>
+        <f>((((((156104.99*($B5-15%)*184/10000)+248.7375+(62629.76*($B5-15%)*10*9/10000))-(1469.87445375+(156104.99*($B5-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B5*365/10000)+396.171+(62629.76*$B5*10*12/10000))-(1955.06445274999+(156104.99*$B5*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B5*366/10000)+463.4658+(62629.76*$B5*10*12/10000))-(1967.0676246285+(156104.99*$B5*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B5*365*(1+C4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+C4)/10000)*2.5%))*75%)+((((156104.99*$B5*365*(1+C4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+C4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>19413.380368266433</v>
       </c>
       <c r="D5" s="37">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B5,敏感性计算明细!$C:$C,D4)</f>
-        <v>20142.198682235656</v>
+        <f>((((((156104.99*($B5-15%)*184/10000)+248.7375+(62629.76*($B5-15%)*10*9/10000))-(1469.87445375+(156104.99*($B5-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B5*365/10000)+396.171+(62629.76*$B5*10*12/10000))-(1955.06445274999+(156104.99*$B5*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B5*366/10000)+463.4658+(62629.76*$B5*10*12/10000))-(1967.0676246285+(156104.99*$B5*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B5*365*(1+D4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+D4)/10000)*2.5%))*75%)+((((156104.99*$B5*365*(1+D4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+D4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>20142.198682235692</v>
       </c>
       <c r="E5" s="38">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B5,敏感性计算明细!$C:$C,E4)</f>
-        <v>20871.016996204911</v>
+        <f>((((((156104.99*($B5-15%)*184/10000)+248.7375+(62629.76*($B5-15%)*10*9/10000))-(1469.87445375+(156104.99*($B5-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B5*365/10000)+396.171+(62629.76*$B5*10*12/10000))-(1955.06445274999+(156104.99*$B5*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B5*366/10000)+463.4658+(62629.76*$B5*10*12/10000))-(1967.0676246285+(156104.99*$B5*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B5*365*(1+E4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+E4)/10000)*2.5%))*75%)+((((156104.99*$B5*365*(1+E4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+E4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>20871.01699620494</v>
       </c>
       <c r="F5" s="39">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B5,敏感性计算明细!$C:$C,F4)</f>
-        <v>21356.895872184403</v>
+        <f>((((((156104.99*($B5-15%)*184/10000)+248.7375+(62629.76*($B5-15%)*10*9/10000))-(1469.87445375+(156104.99*($B5-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B5*365/10000)+396.171+(62629.76*$B5*10*12/10000))-(1955.06445274999+(156104.99*$B5*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B5*366/10000)+463.4658+(62629.76*$B5*10*12/10000))-(1967.0676246285+(156104.99*$B5*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B5*365*(1+F4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+F4)/10000)*2.5%))*75%)+((((156104.99*$B5*365*(1+F4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+F4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>21356.895872184436</v>
       </c>
       <c r="G5" s="40">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B5,敏感性计算明细!$C:$C,G4)</f>
-        <v>22085.714186153647</v>
+        <f>((((((156104.99*($B5-15%)*184/10000)+248.7375+(62629.76*($B5-15%)*10*9/10000))-(1469.87445375+(156104.99*($B5-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B5*365/10000)+396.171+(62629.76*$B5*10*12/10000))-(1955.06445274999+(156104.99*$B5*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B5*366/10000)+463.4658+(62629.76*$B5*10*12/10000))-(1967.0676246285+(156104.99*$B5*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B5*365*(1+G4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+G4)/10000)*2.5%))*75%)+((((156104.99*$B5*365*(1+G4)/10000)+528.228+(62629.76*$B5*10*12/10000))-(1965.79440404631+(156104.99*$B5*365*(1+G4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>22085.714186153687</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="14.65" customHeight="1">
@@ -4491,24 +4525,24 @@
         <v>0.75</v>
       </c>
       <c r="C6" s="41">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B6,敏感性计算明细!$C:$C,C4)</f>
-        <v>21787.607382034643</v>
+        <f>((((((156104.99*($B6-15%)*184/10000)+248.7375+(62629.76*($B6-15%)*10*9/10000))-(1469.87445375+(156104.99*($B6-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B6*365/10000)+396.171+(62629.76*$B6*10*12/10000))-(1955.06445274999+(156104.99*$B6*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B6*366/10000)+463.4658+(62629.76*$B6*10*12/10000))-(1967.0676246285+(156104.99*$B6*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B6*365*(1+C4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+C4)/10000)*2.5%))*75%)+((((156104.99*$B6*365*(1+C4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+C4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>21787.607382034676</v>
       </c>
       <c r="D6" s="42">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B6,敏感性计算明细!$C:$C,D4)</f>
-        <v>22568.484147001691</v>
+        <f>((((((156104.99*($B6-15%)*184/10000)+248.7375+(62629.76*($B6-15%)*10*9/10000))-(1469.87445375+(156104.99*($B6-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B6*365/10000)+396.171+(62629.76*$B6*10*12/10000))-(1955.06445274999+(156104.99*$B6*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B6*366/10000)+463.4658+(62629.76*$B6*10*12/10000))-(1967.0676246285+(156104.99*$B6*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B6*365*(1+D4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+D4)/10000)*2.5%))*75%)+((((156104.99*$B6*365*(1+D4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+D4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>22568.484147001727</v>
       </c>
       <c r="E6" s="43">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B6,敏感性计算明细!$C:$C,E4)</f>
-        <v>23349.360911968743</v>
+        <f>((((((156104.99*($B6-15%)*184/10000)+248.7375+(62629.76*($B6-15%)*10*9/10000))-(1469.87445375+(156104.99*($B6-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B6*365/10000)+396.171+(62629.76*$B6*10*12/10000))-(1955.06445274999+(156104.99*$B6*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B6*366/10000)+463.4658+(62629.76*$B6*10*12/10000))-(1967.0676246285+(156104.99*$B6*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B6*365*(1+E4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+E4)/10000)*2.5%))*75%)+((((156104.99*$B6*365*(1+E4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+E4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>23349.360911968783</v>
       </c>
       <c r="F6" s="44">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B6,敏感性计算明细!$C:$C,F4)</f>
-        <v>23869.945421946781</v>
+        <f>((((((156104.99*($B6-15%)*184/10000)+248.7375+(62629.76*($B6-15%)*10*9/10000))-(1469.87445375+(156104.99*($B6-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B6*365/10000)+396.171+(62629.76*$B6*10*12/10000))-(1955.06445274999+(156104.99*$B6*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B6*366/10000)+463.4658+(62629.76*$B6*10*12/10000))-(1967.0676246285+(156104.99*$B6*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B6*365*(1+F4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+F4)/10000)*2.5%))*75%)+((((156104.99*$B6*365*(1+F4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+F4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>23869.945421946813</v>
       </c>
       <c r="G6" s="45">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B6,敏感性计算明细!$C:$C,G4)</f>
-        <v>24650.822186913829</v>
+        <f>((((((156104.99*($B6-15%)*184/10000)+248.7375+(62629.76*($B6-15%)*10*9/10000))-(1469.87445375+(156104.99*($B6-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B6*365/10000)+396.171+(62629.76*$B6*10*12/10000))-(1955.06445274999+(156104.99*$B6*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B6*366/10000)+463.4658+(62629.76*$B6*10*12/10000))-(1967.0676246285+(156104.99*$B6*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B6*365*(1+G4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+G4)/10000)*2.5%))*75%)+((((156104.99*$B6*365*(1+G4)/10000)+528.228+(62629.76*$B6*10*12/10000))-(1965.79440404631+(156104.99*$B6*365*(1+G4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>24650.822186913862</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="14.65" customHeight="1">
@@ -4516,24 +4550,24 @@
         <v>0.8</v>
       </c>
       <c r="C7" s="46">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B7,敏感性计算明细!$C:$C,C4)</f>
-        <v>24161.834395802871</v>
+        <f>((((((156104.99*($B7-15%)*184/10000)+248.7375+(62629.76*($B7-15%)*10*9/10000))-(1469.87445375+(156104.99*($B7-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B7*365/10000)+396.171+(62629.76*$B7*10*12/10000))-(1955.06445274999+(156104.99*$B7*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B7*366/10000)+463.4658+(62629.76*$B7*10*12/10000))-(1967.0676246285+(156104.99*$B7*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B7*365*(1+C4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+C4)/10000)*2.5%))*75%)+((((156104.99*$B7*365*(1+C4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+C4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>24161.834395802904</v>
       </c>
       <c r="D7" s="47">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B7,敏感性计算明细!$C:$C,D4)</f>
-        <v>24994.769611767726</v>
+        <f>((((((156104.99*($B7-15%)*184/10000)+248.7375+(62629.76*($B7-15%)*10*9/10000))-(1469.87445375+(156104.99*($B7-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B7*365/10000)+396.171+(62629.76*$B7*10*12/10000))-(1955.06445274999+(156104.99*$B7*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B7*366/10000)+463.4658+(62629.76*$B7*10*12/10000))-(1967.0676246285+(156104.99*$B7*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B7*365*(1+D4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+D4)/10000)*2.5%))*75%)+((((156104.99*$B7*365*(1+D4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+D4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>24994.769611767762</v>
       </c>
       <c r="E7" s="48">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B7,敏感性计算明细!$C:$C,E4)</f>
-        <v>25827.704827732588</v>
+        <f>((((((156104.99*($B7-15%)*184/10000)+248.7375+(62629.76*($B7-15%)*10*9/10000))-(1469.87445375+(156104.99*($B7-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B7*365/10000)+396.171+(62629.76*$B7*10*12/10000))-(1955.06445274999+(156104.99*$B7*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B7*366/10000)+463.4658+(62629.76*$B7*10*12/10000))-(1967.0676246285+(156104.99*$B7*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B7*365*(1+E4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+E4)/10000)*2.5%))*75%)+((((156104.99*$B7*365*(1+E4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+E4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>25827.704827732618</v>
       </c>
       <c r="F7" s="49">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B7,敏感性计算明细!$C:$C,F4)</f>
-        <v>26382.994971709159</v>
+        <f>((((((156104.99*($B7-15%)*184/10000)+248.7375+(62629.76*($B7-15%)*10*9/10000))-(1469.87445375+(156104.99*($B7-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B7*365/10000)+396.171+(62629.76*$B7*10*12/10000))-(1955.06445274999+(156104.99*$B7*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B7*366/10000)+463.4658+(62629.76*$B7*10*12/10000))-(1967.0676246285+(156104.99*$B7*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B7*365*(1+F4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+F4)/10000)*2.5%))*75%)+((((156104.99*$B7*365*(1+F4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+F4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>26382.994971709188</v>
       </c>
       <c r="G7" s="50">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B7,敏感性计算明细!$C:$C,G4)</f>
-        <v>27215.930187674014</v>
+        <f>((((((156104.99*($B7-15%)*184/10000)+248.7375+(62629.76*($B7-15%)*10*9/10000))-(1469.87445375+(156104.99*($B7-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B7*365/10000)+396.171+(62629.76*$B7*10*12/10000))-(1955.06445274999+(156104.99*$B7*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B7*366/10000)+463.4658+(62629.76*$B7*10*12/10000))-(1967.0676246285+(156104.99*$B7*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B7*365*(1+G4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+G4)/10000)*2.5%))*75%)+((((156104.99*$B7*365*(1+G4)/10000)+528.228+(62629.76*$B7*10*12/10000))-(1965.79440404631+(156104.99*$B7*365*(1+G4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>27215.930187674054</v>
       </c>
     </row>
     <row r="8" spans="2:7" ht="14.65" customHeight="1">
@@ -4541,24 +4575,24 @@
         <v>0.85</v>
       </c>
       <c r="C8" s="51">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B8,敏感性计算明细!$C:$C,C4)</f>
-        <v>26536.061409571099</v>
+        <f>((((((156104.99*($B8-15%)*184/10000)+248.7375+(62629.76*($B8-15%)*10*9/10000))-(1469.87445375+(156104.99*($B8-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B8*365/10000)+396.171+(62629.76*$B8*10*12/10000))-(1955.06445274999+(156104.99*$B8*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B8*366/10000)+463.4658+(62629.76*$B8*10*12/10000))-(1967.0676246285+(156104.99*$B8*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B8*365*(1+C4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+C4)/10000)*2.5%))*75%)+((((156104.99*$B8*365*(1+C4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+C4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>26536.061409571139</v>
       </c>
       <c r="D8" s="52">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B8,敏感性计算明细!$C:$C,D4)</f>
-        <v>27421.055076533758</v>
+        <f>((((((156104.99*($B8-15%)*184/10000)+248.7375+(62629.76*($B8-15%)*10*9/10000))-(1469.87445375+(156104.99*($B8-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B8*365/10000)+396.171+(62629.76*$B8*10*12/10000))-(1955.06445274999+(156104.99*$B8*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B8*366/10000)+463.4658+(62629.76*$B8*10*12/10000))-(1967.0676246285+(156104.99*$B8*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B8*365*(1+D4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+D4)/10000)*2.5%))*75%)+((((156104.99*$B8*365*(1+D4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+D4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>27421.055076533798</v>
       </c>
       <c r="E8" s="53">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B8,敏感性计算明细!$C:$C,E4)</f>
-        <v>28306.048743496423</v>
+        <f>((((((156104.99*($B8-15%)*184/10000)+248.7375+(62629.76*($B8-15%)*10*9/10000))-(1469.87445375+(156104.99*($B8-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B8*365/10000)+396.171+(62629.76*$B8*10*12/10000))-(1955.06445274999+(156104.99*$B8*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B8*366/10000)+463.4658+(62629.76*$B8*10*12/10000))-(1967.0676246285+(156104.99*$B8*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B8*365*(1+E4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+E4)/10000)*2.5%))*75%)+((((156104.99*$B8*365*(1+E4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+E4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>28306.048743496456</v>
       </c>
       <c r="F8" s="54">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B8,敏感性计算明细!$C:$C,F4)</f>
-        <v>28896.044521471526</v>
+        <f>((((((156104.99*($B8-15%)*184/10000)+248.7375+(62629.76*($B8-15%)*10*9/10000))-(1469.87445375+(156104.99*($B8-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B8*365/10000)+396.171+(62629.76*$B8*10*12/10000))-(1955.06445274999+(156104.99*$B8*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B8*366/10000)+463.4658+(62629.76*$B8*10*12/10000))-(1967.0676246285+(156104.99*$B8*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B8*365*(1+F4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+F4)/10000)*2.5%))*75%)+((((156104.99*$B8*365*(1+F4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+F4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>28896.044521471569</v>
       </c>
       <c r="G8" s="55">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B8,敏感性计算明细!$C:$C,G4)</f>
-        <v>29781.038188434184</v>
+        <f>((((((156104.99*($B8-15%)*184/10000)+248.7375+(62629.76*($B8-15%)*10*9/10000))-(1469.87445375+(156104.99*($B8-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B8*365/10000)+396.171+(62629.76*$B8*10*12/10000))-(1955.06445274999+(156104.99*$B8*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B8*366/10000)+463.4658+(62629.76*$B8*10*12/10000))-(1967.0676246285+(156104.99*$B8*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B8*365*(1+G4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+G4)/10000)*2.5%))*75%)+((((156104.99*$B8*365*(1+G4)/10000)+528.228+(62629.76*$B8*10*12/10000))-(1965.79440404631+(156104.99*$B8*365*(1+G4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>29781.038188434221</v>
       </c>
     </row>
     <row r="9" spans="2:7" ht="14.65" customHeight="1">
@@ -4566,24 +4600,24 @@
         <v>0.9</v>
       </c>
       <c r="C9" s="56">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B9,敏感性计算明细!$C:$C,C4)</f>
-        <v>28910.288423339342</v>
+        <f>((((((156104.99*($B9-15%)*184/10000)+248.7375+(62629.76*($B9-15%)*10*9/10000))-(1469.87445375+(156104.99*($B9-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B9*365/10000)+396.171+(62629.76*$B9*10*12/10000))-(1955.06445274999+(156104.99*$B9*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B9*366/10000)+463.4658+(62629.76*$B9*10*12/10000))-(1967.0676246285+(156104.99*$B9*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B9*365*(1+C4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+C4)/10000)*2.5%))*75%)+((((156104.99*$B9*365*(1+C4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+C4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>28910.288423339378</v>
       </c>
       <c r="D9" s="57">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B9,敏感性计算明细!$C:$C,D4)</f>
-        <v>29847.3405412998</v>
+        <f>((((((156104.99*($B9-15%)*184/10000)+248.7375+(62629.76*($B9-15%)*10*9/10000))-(1469.87445375+(156104.99*($B9-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B9*365/10000)+396.171+(62629.76*$B9*10*12/10000))-(1955.06445274999+(156104.99*$B9*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B9*366/10000)+463.4658+(62629.76*$B9*10*12/10000))-(1967.0676246285+(156104.99*$B9*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B9*365*(1+D4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+D4)/10000)*2.5%))*75%)+((((156104.99*$B9*365*(1+D4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+D4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>29847.340541299844</v>
       </c>
       <c r="E9" s="58">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B9,敏感性计算明细!$C:$C,E4)</f>
-        <v>30784.392659260269</v>
+        <f>((((((156104.99*($B9-15%)*184/10000)+248.7375+(62629.76*($B9-15%)*10*9/10000))-(1469.87445375+(156104.99*($B9-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B9*365/10000)+396.171+(62629.76*$B9*10*12/10000))-(1955.06445274999+(156104.99*$B9*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B9*366/10000)+463.4658+(62629.76*$B9*10*12/10000))-(1967.0676246285+(156104.99*$B9*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B9*365*(1+E4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+E4)/10000)*2.5%))*75%)+((((156104.99*$B9*365*(1+E4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+E4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>30784.392659260298</v>
       </c>
       <c r="F9" s="59">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B9,敏感性计算明细!$C:$C,F4)</f>
-        <v>31409.094071233914</v>
+        <f>((((((156104.99*($B9-15%)*184/10000)+248.7375+(62629.76*($B9-15%)*10*9/10000))-(1469.87445375+(156104.99*($B9-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B9*365/10000)+396.171+(62629.76*$B9*10*12/10000))-(1955.06445274999+(156104.99*$B9*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B9*366/10000)+463.4658+(62629.76*$B9*10*12/10000))-(1967.0676246285+(156104.99*$B9*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B9*365*(1+F4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+F4)/10000)*2.5%))*75%)+((((156104.99*$B9*365*(1+F4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+F4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>31409.094071233943</v>
       </c>
       <c r="G9" s="60">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B9,敏感性计算明细!$C:$C,G4)</f>
-        <v>32346.146189194362</v>
+        <f>((((((156104.99*($B9-15%)*184/10000)+248.7375+(62629.76*($B9-15%)*10*9/10000))-(1469.87445375+(156104.99*($B9-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B9*365/10000)+396.171+(62629.76*$B9*10*12/10000))-(1955.06445274999+(156104.99*$B9*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B9*366/10000)+463.4658+(62629.76*$B9*10*12/10000))-(1967.0676246285+(156104.99*$B9*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B9*365*(1+G4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+G4)/10000)*2.5%))*75%)+((((156104.99*$B9*365*(1+G4)/10000)+528.228+(62629.76*$B9*10*12/10000))-(1965.79440404631+(156104.99*$B9*365*(1+G4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>32346.146189194405</v>
       </c>
     </row>
     <row r="10" spans="2:7" ht="14.65" customHeight="1">
@@ -4591,24 +4625,24 @@
         <v>0.95</v>
       </c>
       <c r="C10" s="61">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B10,敏感性计算明细!$C:$C,C4)</f>
-        <v>31284.515437107562</v>
+        <f>((((((156104.99*($B10-15%)*184/10000)+248.7375+(62629.76*($B10-15%)*10*9/10000))-(1469.87445375+(156104.99*($B10-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B10*365/10000)+396.171+(62629.76*$B10*10*12/10000))-(1955.06445274999+(156104.99*$B10*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B10*366/10000)+463.4658+(62629.76*$B10*10*12/10000))-(1967.0676246285+(156104.99*$B10*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B10*365*(1+C4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+C4)/10000)*2.5%))*75%)+((((156104.99*$B10*365*(1+C4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+C4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>31284.515437107599</v>
       </c>
       <c r="D10" s="62">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B10,敏感性计算明细!$C:$C,D4)</f>
-        <v>32273.626006065828</v>
+        <f>((((((156104.99*($B10-15%)*184/10000)+248.7375+(62629.76*($B10-15%)*10*9/10000))-(1469.87445375+(156104.99*($B10-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B10*365/10000)+396.171+(62629.76*$B10*10*12/10000))-(1955.06445274999+(156104.99*$B10*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B10*366/10000)+463.4658+(62629.76*$B10*10*12/10000))-(1967.0676246285+(156104.99*$B10*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B10*365*(1+D4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+D4)/10000)*2.5%))*75%)+((((156104.99*$B10*365*(1+D4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+D4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>32273.626006065871</v>
       </c>
       <c r="E10" s="22">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B10,敏感性计算明细!$C:$C,E4)</f>
-        <v>33262.736575024093</v>
+        <f>((((((156104.99*($B10-15%)*184/10000)+248.7375+(62629.76*($B10-15%)*10*9/10000))-(1469.87445375+(156104.99*($B10-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B10*365/10000)+396.171+(62629.76*$B10*10*12/10000))-(1955.06445274999+(156104.99*$B10*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B10*366/10000)+463.4658+(62629.76*$B10*10*12/10000))-(1967.0676246285+(156104.99*$B10*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B10*365*(1+E4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+E4)/10000)*2.5%))*75%)+((((156104.99*$B10*365*(1+E4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+E4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>33262.736575024137</v>
       </c>
       <c r="F10" s="63">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B10,敏感性计算明细!$C:$C,F4)</f>
-        <v>33922.143620996278</v>
+        <f>((((((156104.99*($B10-15%)*184/10000)+248.7375+(62629.76*($B10-15%)*10*9/10000))-(1469.87445375+(156104.99*($B10-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B10*365/10000)+396.171+(62629.76*$B10*10*12/10000))-(1955.06445274999+(156104.99*$B10*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B10*366/10000)+463.4658+(62629.76*$B10*10*12/10000))-(1967.0676246285+(156104.99*$B10*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B10*365*(1+F4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+F4)/10000)*2.5%))*75%)+((((156104.99*$B10*365*(1+F4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+F4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>33922.143620996307</v>
       </c>
       <c r="G10" s="64">
-        <f>SUMIFS(敏感性计算明细!$AM:$AM,敏感性计算明细!$B:$B,$B10,敏感性计算明细!$C:$C,G4)</f>
-        <v>34911.254189954539</v>
+        <f>((((((156104.99*($B10-15%)*184/10000)+248.7375+(62629.76*($B10-15%)*10*9/10000))-(1469.87445375+(156104.99*($B10-15%)*184/10000)*2.5%))*75%)/(1+12%)^1+((((156104.99*$B10*365/10000)+396.171+(62629.76*$B10*10*12/10000))-(1955.06445274999+(156104.99*$B10*365/10000)*2.5%))*75%)/(1+12%)^2+((((156104.99*$B10*366/10000)+463.4658+(62629.76*$B10*10*12/10000))-(1967.0676246285+(156104.99*$B10*366/10000)*2.5%))*75%)/(1+12%)^3+(((((156104.99*$B10*365*(1+G4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+G4)/10000)*2.5%))*75%)+((((156104.99*$B10*365*(1+G4)/10000)+528.228+(62629.76*$B10*10*12/10000))-(1965.79440404631+(156104.99*$B10*365*(1+G4)/10000)*2.5%))*75%)/8%)/(1+12%)^4)-1100-1000)/(1+3%)</f>
+        <v>34911.254189954569</v>
       </c>
     </row>
     <row r="11" spans="2:7">
@@ -4649,11 +4683,11 @@
       </c>
       <c r="C14" s="14">
         <f t="shared" ref="C14:C19" si="0">E5</f>
-        <v>20871.016996204911</v>
+        <v>20871.01699620494</v>
       </c>
       <c r="D14" s="65">
         <f t="shared" ref="D14:D19" si="1">(C14-$E$10)/$E$10</f>
-        <v>-0.37254059210882007</v>
+        <v>-0.37254059210882001</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="3"/>
@@ -4665,11 +4699,11 @@
       </c>
       <c r="C15" s="14">
         <f t="shared" si="0"/>
-        <v>23349.360911968743</v>
+        <v>23349.360911968783</v>
       </c>
       <c r="D15" s="65">
         <f t="shared" si="1"/>
-        <v>-0.29803247368705621</v>
+        <v>-0.29803247368705593</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -4681,11 +4715,11 @@
       </c>
       <c r="C16" s="14">
         <f t="shared" si="0"/>
-        <v>25827.704827732588</v>
+        <v>25827.704827732618</v>
       </c>
       <c r="D16" s="65">
         <f t="shared" si="1"/>
-        <v>-0.22352435526529194</v>
+        <v>-0.22352435526529207</v>
       </c>
       <c r="E16" s="3"/>
       <c r="F16" s="3"/>
@@ -4697,11 +4731,11 @@
       </c>
       <c r="C17" s="14">
         <f t="shared" si="0"/>
-        <v>28306.048743496423</v>
+        <v>28306.048743496456</v>
       </c>
       <c r="D17" s="65">
         <f t="shared" si="1"/>
-        <v>-0.14901623684352794</v>
+        <v>-0.14901623684352808</v>
       </c>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -4713,11 +4747,11 @@
       </c>
       <c r="C18" s="14">
         <f t="shared" si="0"/>
-        <v>30784.392659260269</v>
+        <v>30784.392659260298</v>
       </c>
       <c r="D18" s="65">
         <f t="shared" si="1"/>
-        <v>-7.450811842176365E-2</v>
+        <v>-7.4508118421763983E-2</v>
       </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -4729,7 +4763,7 @@
       </c>
       <c r="C19" s="20">
         <f t="shared" si="0"/>
-        <v>33262.736575024093</v>
+        <v>33262.736575024137</v>
       </c>
       <c r="D19" s="66">
         <f t="shared" si="1"/>
@@ -4777,11 +4811,11 @@
       </c>
       <c r="C23" s="14">
         <f>C10</f>
-        <v>31284.515437107562</v>
+        <v>31284.515437107599</v>
       </c>
       <c r="D23" s="65">
         <f>(C23-$E$10)/$E$10</f>
-        <v>-5.9472591302121333E-2</v>
+        <v>-5.9472591302121472E-2</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -4793,11 +4827,11 @@
       </c>
       <c r="C24" s="14">
         <f>D10</f>
-        <v>32273.626006065828</v>
+        <v>32273.626006065871</v>
       </c>
       <c r="D24" s="65">
         <f>(C24-$E$10)/$E$10</f>
-        <v>-2.9736295651060667E-2</v>
+        <v>-2.9736295651060628E-2</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3"/>
@@ -4809,7 +4843,7 @@
       </c>
       <c r="C25" s="20">
         <f>E10</f>
-        <v>33262.736575024093</v>
+        <v>33262.736575024137</v>
       </c>
       <c r="D25" s="66">
         <f>(C25-$E$10)/$E$10</f>
@@ -4825,11 +4859,11 @@
       </c>
       <c r="C26" s="14">
         <f>F10</f>
-        <v>33922.143620996278</v>
+        <v>33922.143620996307</v>
       </c>
       <c r="D26" s="66">
         <f>(C26-$E$10)/$E$10</f>
-        <v>1.982419710070733E-2</v>
+        <v>1.9824197100706865E-2</v>
       </c>
       <c r="E26" s="3"/>
       <c r="F26" s="3"/>
@@ -4841,11 +4875,11 @@
       </c>
       <c r="C27" s="14">
         <f>G10</f>
-        <v>34911.254189954539</v>
+        <v>34911.254189954569</v>
       </c>
       <c r="D27" s="66">
         <f>(C27-$E$10)/$E$10</f>
-        <v>4.9560492751767889E-2</v>
+        <v>4.9560492751767382E-2</v>
       </c>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
@@ -4878,9 +4912,8 @@
       <c r="G30" s="91"/>
     </row>
     <row r="31" spans="2:7" ht="34.049999999999997" customHeight="1">
-      <c r="B31" s="102" t="str">
-        <f>"基准假设（出租率95%，租金增长率3%）下建议收购价约 "&amp;TEXT($E$10,"0")&amp;" 万元（3.33亿元）。按“2026年出租率=稳定期出租率-15个百分点”的口径，出租率每下降5个百分点，收购对价约下降"&amp;TEXT($E$10-$E$9,"0")&amp;"万元；若稳定出租率仅70%且2029年租金增长率为-3%，合理价格约"&amp;TEXT($C$5,"0")&amp;"万元。"</f>
-        <v>基准假设（出租率95%，租金增长率3%）下建议收购价约 33263 万元（3.33亿元）。按“2026年出租率=稳定期出租率-15个百分点”的口径，出租率每下降5个百分点，收购对价约下降2478万元；若稳定出租率仅70%且2029年租金增长率为-3%，合理价格约19413万元。</v>
+      <c r="B31" s="102" t="s">
+        <v>188</v>
       </c>
       <c r="C31" s="103"/>
       <c r="D31" s="103"/>
@@ -4914,7 +4947,8 @@
     <mergeCell ref="B21:G21"/>
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.25" right="0.25" top="0.35" bottom="0.35" header="0.15" footer="0.15"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -4930,9 +4964,9 @@
     <col min="39" max="39" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" ht="18.399999999999999">
+    <row r="1" spans="1:39" ht="18.399999999999999" customHeight="1">
       <c r="A1" s="110" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B1" s="88"/>
       <c r="C1" s="88"/>
@@ -4975,126 +5009,126 @@
     </row>
     <row r="3" spans="1:39">
       <c r="A3" s="82" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B3" s="82" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C3" s="82" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D3" s="82" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="E3" s="82" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="F3" s="82" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="G3" s="82" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="H3" s="82" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I3" s="82" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="J3" s="82" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K3" s="82" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L3" s="82" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="M3" s="82" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="N3" s="82" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="O3" s="82" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P3" s="82" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Q3" s="82" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="R3" s="82" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="S3" s="82" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="T3" s="82" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="U3" s="82" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="V3" s="82" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="W3" s="82" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="X3" s="82" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Y3" s="82" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Z3" s="82" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="AA3" s="82" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AB3" s="82" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="AC3" s="82" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AD3" s="82" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AE3" s="82" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AF3" s="82" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AG3" s="82" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="AH3" s="82" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AI3" s="82" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AJ3" s="82" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="AK3" s="82" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="AL3" s="82" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="AM3" s="82" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:39">
       <c r="A4" s="83" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B4" s="84">
         <v>0.7</v>
@@ -5249,7 +5283,7 @@
     </row>
     <row r="5" spans="1:39">
       <c r="A5" s="83" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B5" s="84">
         <v>0.7</v>
@@ -5404,7 +5438,7 @@
     </row>
     <row r="6" spans="1:39">
       <c r="A6" s="83" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B6" s="84">
         <v>0.7</v>
@@ -5559,7 +5593,7 @@
     </row>
     <row r="7" spans="1:39">
       <c r="A7" s="83" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B7" s="84">
         <v>0.7</v>
@@ -5714,7 +5748,7 @@
     </row>
     <row r="8" spans="1:39">
       <c r="A8" s="83" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B8" s="84">
         <v>0.7</v>
@@ -5869,7 +5903,7 @@
     </row>
     <row r="9" spans="1:39">
       <c r="A9" s="83" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B9" s="84">
         <v>0.75</v>
@@ -6024,7 +6058,7 @@
     </row>
     <row r="10" spans="1:39">
       <c r="A10" s="83" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B10" s="84">
         <v>0.75</v>
@@ -6179,7 +6213,7 @@
     </row>
     <row r="11" spans="1:39">
       <c r="A11" s="83" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B11" s="84">
         <v>0.75</v>
@@ -6334,7 +6368,7 @@
     </row>
     <row r="12" spans="1:39">
       <c r="A12" s="83" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B12" s="84">
         <v>0.75</v>
@@ -6489,7 +6523,7 @@
     </row>
     <row r="13" spans="1:39">
       <c r="A13" s="83" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B13" s="84">
         <v>0.75</v>
@@ -6644,7 +6678,7 @@
     </row>
     <row r="14" spans="1:39">
       <c r="A14" s="83" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B14" s="84">
         <v>0.8</v>
@@ -6799,7 +6833,7 @@
     </row>
     <row r="15" spans="1:39">
       <c r="A15" s="83" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B15" s="84">
         <v>0.8</v>
@@ -6954,7 +6988,7 @@
     </row>
     <row r="16" spans="1:39">
       <c r="A16" s="83" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B16" s="84">
         <v>0.8</v>
@@ -7109,7 +7143,7 @@
     </row>
     <row r="17" spans="1:39">
       <c r="A17" s="83" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B17" s="84">
         <v>0.8</v>
@@ -7264,7 +7298,7 @@
     </row>
     <row r="18" spans="1:39">
       <c r="A18" s="83" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B18" s="84">
         <v>0.8</v>
@@ -7419,7 +7453,7 @@
     </row>
     <row r="19" spans="1:39">
       <c r="A19" s="83" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B19" s="84">
         <v>0.85</v>
@@ -7574,7 +7608,7 @@
     </row>
     <row r="20" spans="1:39">
       <c r="A20" s="83" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B20" s="84">
         <v>0.85</v>
@@ -7729,7 +7763,7 @@
     </row>
     <row r="21" spans="1:39">
       <c r="A21" s="83" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B21" s="84">
         <v>0.85</v>
@@ -7884,7 +7918,7 @@
     </row>
     <row r="22" spans="1:39">
       <c r="A22" s="83" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B22" s="84">
         <v>0.85</v>
@@ -8039,7 +8073,7 @@
     </row>
     <row r="23" spans="1:39">
       <c r="A23" s="83" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B23" s="84">
         <v>0.85</v>
@@ -8194,7 +8228,7 @@
     </row>
     <row r="24" spans="1:39">
       <c r="A24" s="83" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B24" s="84">
         <v>0.9</v>
@@ -8349,7 +8383,7 @@
     </row>
     <row r="25" spans="1:39">
       <c r="A25" s="83" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B25" s="84">
         <v>0.9</v>
@@ -8504,7 +8538,7 @@
     </row>
     <row r="26" spans="1:39">
       <c r="A26" s="83" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B26" s="84">
         <v>0.9</v>
@@ -8659,7 +8693,7 @@
     </row>
     <row r="27" spans="1:39">
       <c r="A27" s="83" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B27" s="84">
         <v>0.9</v>
@@ -8814,7 +8848,7 @@
     </row>
     <row r="28" spans="1:39">
       <c r="A28" s="83" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B28" s="84">
         <v>0.9</v>
@@ -8969,7 +9003,7 @@
     </row>
     <row r="29" spans="1:39">
       <c r="A29" s="83" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B29" s="84">
         <v>0.95</v>
@@ -9124,7 +9158,7 @@
     </row>
     <row r="30" spans="1:39">
       <c r="A30" s="83" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B30" s="84">
         <v>0.95</v>
@@ -9279,7 +9313,7 @@
     </row>
     <row r="31" spans="1:39">
       <c r="A31" s="83" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B31" s="84">
         <v>0.95</v>
@@ -9434,7 +9468,7 @@
     </row>
     <row r="32" spans="1:39">
       <c r="A32" s="83" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B32" s="84">
         <v>0.95</v>
@@ -9589,7 +9623,7 @@
     </row>
     <row r="33" spans="1:39">
       <c r="A33" s="83" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B33" s="84">
         <v>0.95</v>

</xml_diff>

<commit_message>
Polish workbook review details
</commit_message>
<xml_diff>
--- a/final_report/宁波怡丰汇投资分析.xlsx
+++ b/final_report/宁波怡丰汇投资分析.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\课程文件\工程经济学\case_study\EngineringEconomyCaseStudy\final_report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95E6654D-3280-4AD4-9DBB-2CC102C6D405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13AF29E-8480-4B5F-8045-129F16D24345}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3308" yWindow="3308" windowWidth="21600" windowHeight="11332" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,13 +29,14 @@
     <definedName name="_xlnm.Print_Area" localSheetId="2">年度现金流!$B$1:$G$34</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">收购价格!$B$1:$F$30</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">主要假设!$B$1:$H$64</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">敏感性计算明细!$A:$D</definedName>
   </definedNames>
   <calcPr calcId="191029" forceFullCalc="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="258">
   <si>
     <t>宁波怡丰汇商业项目</t>
   </si>
@@ -151,7 +152,7 @@
     <t>出租率</t>
   </si>
   <si>
-    <t>租金增长率（vs上年）</t>
+    <t>租金增长率（较上年）</t>
   </si>
   <si>
     <t>租金收取天数</t>
@@ -443,7 +444,7 @@
     <t>Q3 = Q4（2026）：同等运营条件，现金流基本持平</t>
   </si>
   <si>
-    <t>改造期年度净CF（2026）≈ 1103万元  vs  稳定期（2027）≈ 3325万元，相差约2222万元（约202%增幅）</t>
+    <t>改造期年度净CF（2026）≈ 1103万元，相较稳定期（2027）≈ 3325万元，相差约2222万元（约202%增幅）</t>
   </si>
   <si>
     <t>Step 2：收购价格估算（MARR = 12%）</t>
@@ -542,10 +543,7 @@
     <t>总投资回报倍数（含退出价值）</t>
   </si>
   <si>
-    <t>退出价值 / 总现金流入</t>
-  </si>
-  <si>
-    <t>%</t>
+    <t>退出价值 / 总投资额</t>
   </si>
   <si>
     <t>总CF现值 / 总投资</t>
@@ -566,7 +564,7 @@
     <t>收购价格（万元）</t>
   </si>
   <si>
-    <t>vs基准（95%, 3%）</t>
+    <t>相较基准（95%, 3%）</t>
   </si>
   <si>
     <t>70%</t>
@@ -1370,7 +1368,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1618,6 +1616,9 @@
     </xf>
     <xf numFmtId="0" fontId="23" fillId="42" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="9" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1988,15 +1989,15 @@
   <sheetData>
     <row r="1" spans="2:2" ht="40.049999999999997" customHeight="1"/>
     <row r="2" spans="2:2">
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="88" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="2:2">
-      <c r="B3" s="88"/>
+      <c r="B3" s="89"/>
     </row>
     <row r="4" spans="2:2" ht="18.399999999999999" customHeight="1">
-      <c r="B4" s="86" t="s">
+      <c r="B4" s="87" t="s">
         <v>1</v>
       </c>
     </row>
@@ -2063,15 +2064,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="18.399999999999999" customHeight="1">
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="93" t="s">
         <v>9</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="90"/>
-      <c r="H1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="91"/>
+      <c r="H1" s="92"/>
     </row>
     <row r="2" spans="2:8">
       <c r="B2" s="3"/>
@@ -2083,15 +2084,15 @@
       <c r="H2" s="3"/>
     </row>
     <row r="3" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B3" s="89" t="s">
+      <c r="B3" s="90" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="90"/>
-      <c r="H3" s="91"/>
+      <c r="C3" s="91"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="91"/>
+      <c r="H3" s="92"/>
     </row>
     <row r="4" spans="2:8" ht="14.65" customHeight="1">
       <c r="B4" s="4" t="s">
@@ -2318,15 +2319,15 @@
       <c r="H14" s="3"/>
     </row>
     <row r="15" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B15" s="89" t="s">
+      <c r="B15" s="90" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="90"/>
-      <c r="D15" s="90"/>
-      <c r="E15" s="90"/>
-      <c r="F15" s="90"/>
-      <c r="G15" s="90"/>
-      <c r="H15" s="91"/>
+      <c r="C15" s="91"/>
+      <c r="D15" s="91"/>
+      <c r="E15" s="91"/>
+      <c r="F15" s="91"/>
+      <c r="G15" s="91"/>
+      <c r="H15" s="92"/>
     </row>
     <row r="16" spans="2:8" ht="13.9" customHeight="1">
       <c r="B16" s="5" t="s">
@@ -2442,15 +2443,15 @@
       <c r="H24" s="3"/>
     </row>
     <row r="25" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B25" s="89" t="s">
+      <c r="B25" s="90" t="s">
         <v>35</v>
       </c>
-      <c r="C25" s="90"/>
-      <c r="D25" s="90"/>
-      <c r="E25" s="90"/>
-      <c r="F25" s="90"/>
-      <c r="G25" s="90"/>
-      <c r="H25" s="91"/>
+      <c r="C25" s="91"/>
+      <c r="D25" s="91"/>
+      <c r="E25" s="91"/>
+      <c r="F25" s="91"/>
+      <c r="G25" s="91"/>
+      <c r="H25" s="92"/>
     </row>
     <row r="26" spans="2:8" ht="24" customHeight="1">
       <c r="B26" s="4" t="s">
@@ -2557,15 +2558,15 @@
       <c r="H31" s="3"/>
     </row>
     <row r="32" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B32" s="89" t="s">
+      <c r="B32" s="90" t="s">
         <v>45</v>
       </c>
-      <c r="C32" s="90"/>
-      <c r="D32" s="90"/>
-      <c r="E32" s="90"/>
-      <c r="F32" s="90"/>
-      <c r="G32" s="90"/>
-      <c r="H32" s="91"/>
+      <c r="C32" s="91"/>
+      <c r="D32" s="91"/>
+      <c r="E32" s="91"/>
+      <c r="F32" s="91"/>
+      <c r="G32" s="91"/>
+      <c r="H32" s="92"/>
     </row>
     <row r="33" spans="2:8" ht="24" customHeight="1">
       <c r="B33" s="4" t="s">
@@ -2662,15 +2663,15 @@
       <c r="H38" s="3"/>
     </row>
     <row r="39" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B39" s="89" t="s">
+      <c r="B39" s="90" t="s">
         <v>49</v>
       </c>
-      <c r="C39" s="90"/>
-      <c r="D39" s="90"/>
-      <c r="E39" s="90"/>
-      <c r="F39" s="90"/>
-      <c r="G39" s="90"/>
-      <c r="H39" s="91"/>
+      <c r="C39" s="91"/>
+      <c r="D39" s="91"/>
+      <c r="E39" s="91"/>
+      <c r="F39" s="91"/>
+      <c r="G39" s="91"/>
+      <c r="H39" s="92"/>
     </row>
     <row r="40" spans="2:8" ht="13.9" customHeight="1">
       <c r="B40" s="12" t="s">
@@ -2787,15 +2788,15 @@
       <c r="H47" s="3"/>
     </row>
     <row r="48" spans="2:8" ht="24" customHeight="1">
-      <c r="B48" s="89" t="s">
+      <c r="B48" s="90" t="s">
         <v>60</v>
       </c>
-      <c r="C48" s="90"/>
-      <c r="D48" s="90"/>
-      <c r="E48" s="90"/>
-      <c r="F48" s="90"/>
-      <c r="G48" s="90"/>
-      <c r="H48" s="91"/>
+      <c r="C48" s="91"/>
+      <c r="D48" s="91"/>
+      <c r="E48" s="91"/>
+      <c r="F48" s="91"/>
+      <c r="G48" s="91"/>
+      <c r="H48" s="92"/>
     </row>
     <row r="49" spans="2:8" ht="14.65" customHeight="1">
       <c r="B49" s="4" t="s">
@@ -2940,15 +2941,15 @@
       <c r="H56" s="3"/>
     </row>
     <row r="57" spans="2:8" ht="15.75" customHeight="1">
-      <c r="B57" s="89" t="s">
+      <c r="B57" s="90" t="s">
         <v>64</v>
       </c>
-      <c r="C57" s="90"/>
-      <c r="D57" s="90"/>
-      <c r="E57" s="90"/>
-      <c r="F57" s="90"/>
-      <c r="G57" s="90"/>
-      <c r="H57" s="91"/>
+      <c r="C57" s="91"/>
+      <c r="D57" s="91"/>
+      <c r="E57" s="91"/>
+      <c r="F57" s="91"/>
+      <c r="G57" s="91"/>
+      <c r="H57" s="92"/>
     </row>
     <row r="58" spans="2:8" ht="13.9" customHeight="1">
       <c r="B58" s="12" t="s">
@@ -3095,24 +3096,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18.399999999999999" customHeight="1">
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="93" t="s">
         <v>78</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="92"/>
     </row>
     <row r="2" spans="2:7">
-      <c r="B2" s="94" t="s">
+      <c r="B2" s="95" t="s">
         <v>79</v>
       </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="92"/>
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="3"/>
@@ -3143,14 +3144,14 @@
       </c>
     </row>
     <row r="5" spans="2:7" ht="14.65" customHeight="1">
-      <c r="B5" s="93" t="s">
+      <c r="B5" s="94" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="90"/>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="90"/>
-      <c r="G5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="91"/>
+      <c r="G5" s="92"/>
     </row>
     <row r="6" spans="2:7" ht="13.9" customHeight="1">
       <c r="B6" s="12" t="s">
@@ -3241,14 +3242,14 @@
       <c r="G9" s="3"/>
     </row>
     <row r="10" spans="2:7" ht="14.65" customHeight="1">
-      <c r="B10" s="96" t="s">
+      <c r="B10" s="97" t="s">
         <v>91</v>
       </c>
-      <c r="C10" s="90"/>
-      <c r="D10" s="90"/>
-      <c r="E10" s="90"/>
-      <c r="F10" s="90"/>
-      <c r="G10" s="91"/>
+      <c r="C10" s="91"/>
+      <c r="D10" s="91"/>
+      <c r="E10" s="91"/>
+      <c r="F10" s="91"/>
+      <c r="G10" s="92"/>
     </row>
     <row r="11" spans="2:7" ht="13.9" customHeight="1">
       <c r="B11" s="12" t="s">
@@ -3427,14 +3428,14 @@
       <c r="G18" s="3"/>
     </row>
     <row r="19" spans="2:7" ht="14.65" customHeight="1">
-      <c r="B19" s="95" t="s">
+      <c r="B19" s="96" t="s">
         <v>100</v>
       </c>
-      <c r="C19" s="90"/>
-      <c r="D19" s="90"/>
-      <c r="E19" s="90"/>
-      <c r="F19" s="90"/>
-      <c r="G19" s="91"/>
+      <c r="C19" s="91"/>
+      <c r="D19" s="91"/>
+      <c r="E19" s="91"/>
+      <c r="F19" s="91"/>
+      <c r="G19" s="92"/>
     </row>
     <row r="20" spans="2:7" ht="14.65" customHeight="1">
       <c r="B20" s="19" t="s">
@@ -3503,14 +3504,14 @@
       <c r="G22" s="3"/>
     </row>
     <row r="23" spans="2:7" ht="14.65" customHeight="1">
-      <c r="B23" s="98" t="s">
+      <c r="B23" s="99" t="s">
         <v>104</v>
       </c>
-      <c r="C23" s="90"/>
-      <c r="D23" s="90"/>
-      <c r="E23" s="90"/>
-      <c r="F23" s="90"/>
-      <c r="G23" s="91"/>
+      <c r="C23" s="91"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="92"/>
     </row>
     <row r="24" spans="2:7" ht="14.65" customHeight="1">
       <c r="B24" s="23" t="s">
@@ -3526,14 +3527,14 @@
       <c r="G24" s="3"/>
     </row>
     <row r="25" spans="2:7" ht="14.65" customHeight="1">
-      <c r="B25" s="93" t="s">
+      <c r="B25" s="94" t="s">
         <v>106</v>
       </c>
-      <c r="C25" s="90"/>
-      <c r="D25" s="90"/>
-      <c r="E25" s="90"/>
-      <c r="F25" s="90"/>
-      <c r="G25" s="91"/>
+      <c r="C25" s="91"/>
+      <c r="D25" s="91"/>
+      <c r="E25" s="91"/>
+      <c r="F25" s="91"/>
+      <c r="G25" s="92"/>
     </row>
     <row r="26" spans="2:7" ht="14.65" customHeight="1">
       <c r="B26" s="15" t="s">
@@ -3566,14 +3567,14 @@
       <c r="G27" s="3"/>
     </row>
     <row r="28" spans="2:7" ht="15.75" customHeight="1">
-      <c r="B28" s="97" t="s">
+      <c r="B28" s="98" t="s">
         <v>108</v>
       </c>
-      <c r="C28" s="90"/>
-      <c r="D28" s="90"/>
-      <c r="E28" s="90"/>
-      <c r="F28" s="90"/>
-      <c r="G28" s="91"/>
+      <c r="C28" s="91"/>
+      <c r="D28" s="91"/>
+      <c r="E28" s="91"/>
+      <c r="F28" s="91"/>
+      <c r="G28" s="92"/>
     </row>
     <row r="29" spans="2:7" ht="13.9" customHeight="1">
       <c r="B29" s="12" t="s">
@@ -3702,22 +3703,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:6" ht="18.399999999999999" customHeight="1">
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="93" t="s">
         <v>112</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="92"/>
     </row>
     <row r="2" spans="2:6">
-      <c r="B2" s="94" t="s">
+      <c r="B2" s="95" t="s">
         <v>113</v>
       </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="92"/>
     </row>
     <row r="3" spans="2:6">
       <c r="B3" s="3"/>
@@ -3744,13 +3745,13 @@
       </c>
     </row>
     <row r="5" spans="2:6" ht="14.65" customHeight="1">
-      <c r="B5" s="93" t="s">
+      <c r="B5" s="94" t="s">
         <v>118</v>
       </c>
-      <c r="C5" s="90"/>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="92"/>
     </row>
     <row r="6" spans="2:6" ht="13.9" customHeight="1">
       <c r="B6" s="26" t="s">
@@ -3834,13 +3835,13 @@
       </c>
     </row>
     <row r="10" spans="2:6" ht="14.65" customHeight="1">
-      <c r="B10" s="96" t="s">
+      <c r="B10" s="97" t="s">
         <v>123</v>
       </c>
-      <c r="C10" s="90"/>
-      <c r="D10" s="90"/>
-      <c r="E10" s="90"/>
-      <c r="F10" s="91"/>
+      <c r="C10" s="91"/>
+      <c r="D10" s="91"/>
+      <c r="E10" s="91"/>
+      <c r="F10" s="92"/>
     </row>
     <row r="11" spans="2:6" ht="13.9" customHeight="1">
       <c r="B11" s="28" t="s">
@@ -3864,13 +3865,13 @@
       </c>
     </row>
     <row r="12" spans="2:6" ht="14.65" customHeight="1">
-      <c r="B12" s="95" t="s">
+      <c r="B12" s="96" t="s">
         <v>125</v>
       </c>
-      <c r="C12" s="90"/>
-      <c r="D12" s="90"/>
-      <c r="E12" s="90"/>
-      <c r="F12" s="91"/>
+      <c r="C12" s="91"/>
+      <c r="D12" s="91"/>
+      <c r="E12" s="91"/>
+      <c r="F12" s="92"/>
     </row>
     <row r="13" spans="2:6" ht="14.65" customHeight="1">
       <c r="B13" s="21" t="s">
@@ -3901,13 +3902,13 @@
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="2:6" ht="14.65" customHeight="1">
-      <c r="B15" s="101" t="s">
+      <c r="B15" s="102" t="s">
         <v>127</v>
       </c>
-      <c r="C15" s="90"/>
-      <c r="D15" s="90"/>
-      <c r="E15" s="90"/>
-      <c r="F15" s="91"/>
+      <c r="C15" s="91"/>
+      <c r="D15" s="91"/>
+      <c r="E15" s="91"/>
+      <c r="F15" s="92"/>
     </row>
     <row r="16" spans="2:6" ht="29.25" customHeight="1">
       <c r="B16" s="23" t="s">
@@ -3942,49 +3943,49 @@
       <c r="F18" s="3"/>
     </row>
     <row r="19" spans="2:6" ht="14.65" customHeight="1">
-      <c r="B19" s="101" t="s">
+      <c r="B19" s="102" t="s">
         <v>130</v>
       </c>
-      <c r="C19" s="90"/>
-      <c r="D19" s="90"/>
-      <c r="E19" s="90"/>
-      <c r="F19" s="91"/>
+      <c r="C19" s="91"/>
+      <c r="D19" s="91"/>
+      <c r="E19" s="91"/>
+      <c r="F19" s="92"/>
     </row>
     <row r="20" spans="2:6" ht="30" customHeight="1">
-      <c r="B20" s="100" t="s">
+      <c r="B20" s="101" t="s">
         <v>131</v>
       </c>
-      <c r="C20" s="90"/>
-      <c r="D20" s="90"/>
-      <c r="E20" s="90"/>
-      <c r="F20" s="91"/>
+      <c r="C20" s="91"/>
+      <c r="D20" s="91"/>
+      <c r="E20" s="91"/>
+      <c r="F20" s="92"/>
     </row>
     <row r="21" spans="2:6" ht="30" customHeight="1">
-      <c r="B21" s="100" t="s">
+      <c r="B21" s="101" t="s">
         <v>132</v>
       </c>
-      <c r="C21" s="90"/>
-      <c r="D21" s="90"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="91"/>
+      <c r="C21" s="91"/>
+      <c r="D21" s="91"/>
+      <c r="E21" s="91"/>
+      <c r="F21" s="92"/>
     </row>
     <row r="22" spans="2:6" ht="24" customHeight="1">
-      <c r="B22" s="100" t="s">
+      <c r="B22" s="101" t="s">
         <v>133</v>
       </c>
-      <c r="C22" s="90"/>
-      <c r="D22" s="90"/>
-      <c r="E22" s="90"/>
-      <c r="F22" s="91"/>
+      <c r="C22" s="91"/>
+      <c r="D22" s="91"/>
+      <c r="E22" s="91"/>
+      <c r="F22" s="92"/>
     </row>
     <row r="23" spans="2:6" ht="38" customHeight="1">
-      <c r="B23" s="99" t="s">
+      <c r="B23" s="100" t="s">
         <v>134</v>
       </c>
-      <c r="C23" s="90"/>
-      <c r="D23" s="90"/>
-      <c r="E23" s="90"/>
-      <c r="F23" s="91"/>
+      <c r="C23" s="91"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="92"/>
     </row>
     <row r="24" spans="2:6">
       <c r="B24" s="3"/>
@@ -4031,14 +4032,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18.399999999999999" customHeight="1">
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="93" t="s">
         <v>135</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="91"/>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="92"/>
     </row>
     <row r="2" spans="2:7">
       <c r="B2" s="3"/>
@@ -4049,14 +4050,14 @@
       <c r="G2" s="3"/>
     </row>
     <row r="3" spans="2:7" ht="15.75" customHeight="1">
-      <c r="B3" s="89" t="s">
+      <c r="B3" s="90" t="s">
         <v>136</v>
       </c>
-      <c r="C3" s="90"/>
-      <c r="D3" s="90"/>
-      <c r="E3" s="90"/>
-      <c r="F3" s="90"/>
-      <c r="G3" s="91"/>
+      <c r="C3" s="91"/>
+      <c r="D3" s="91"/>
+      <c r="E3" s="91"/>
+      <c r="F3" s="91"/>
+      <c r="G3" s="92"/>
     </row>
     <row r="4" spans="2:7" ht="14.65" customHeight="1">
       <c r="B4" s="67" t="s">
@@ -4182,14 +4183,14 @@
       <c r="G10" s="3"/>
     </row>
     <row r="11" spans="2:7" ht="15.75" customHeight="1">
-      <c r="B11" s="89" t="s">
+      <c r="B11" s="90" t="s">
         <v>150</v>
       </c>
-      <c r="C11" s="90"/>
-      <c r="D11" s="90"/>
-      <c r="E11" s="90"/>
-      <c r="F11" s="90"/>
-      <c r="G11" s="91"/>
+      <c r="C11" s="91"/>
+      <c r="D11" s="91"/>
+      <c r="E11" s="91"/>
+      <c r="F11" s="91"/>
+      <c r="G11" s="92"/>
     </row>
     <row r="12" spans="2:7" ht="13.9" customHeight="1">
       <c r="B12" s="12" t="s">
@@ -4350,14 +4351,14 @@
       <c r="G22" s="3"/>
     </row>
     <row r="23" spans="2:7" ht="15.75" customHeight="1">
-      <c r="B23" s="89" t="s">
+      <c r="B23" s="90" t="s">
         <v>162</v>
       </c>
-      <c r="C23" s="90"/>
-      <c r="D23" s="90"/>
-      <c r="E23" s="90"/>
-      <c r="F23" s="90"/>
-      <c r="G23" s="91"/>
+      <c r="C23" s="91"/>
+      <c r="D23" s="91"/>
+      <c r="E23" s="91"/>
+      <c r="F23" s="91"/>
+      <c r="G23" s="92"/>
     </row>
     <row r="24" spans="2:7" ht="14.65" customHeight="1">
       <c r="B24" s="12" t="s">
@@ -4408,20 +4409,18 @@
       <c r="B27" s="12" t="s">
         <v>167</v>
       </c>
-      <c r="C27" s="35">
+      <c r="C27" s="86">
         <f>44178.359863582/C21</f>
         <v>1.2150057253362496</v>
       </c>
-      <c r="D27" s="12" t="s">
-        <v>168</v>
-      </c>
+      <c r="D27" s="12"/>
       <c r="E27" s="3"/>
       <c r="F27" s="3"/>
       <c r="G27" s="3"/>
     </row>
     <row r="28" spans="2:7" ht="14.65" customHeight="1">
       <c r="B28" s="12" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C28" s="35">
         <f>F9/C21</f>
@@ -4477,24 +4476,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:7" ht="18.399999999999999" customHeight="1">
-      <c r="B1" s="92" t="s">
+      <c r="B1" s="93" t="s">
+        <v>169</v>
+      </c>
+      <c r="C1" s="91"/>
+      <c r="D1" s="91"/>
+      <c r="E1" s="91"/>
+      <c r="F1" s="91"/>
+      <c r="G1" s="92"/>
+    </row>
+    <row r="2" spans="2:7">
+      <c r="B2" s="95" t="s">
         <v>170</v>
       </c>
-      <c r="C1" s="90"/>
-      <c r="D1" s="90"/>
-      <c r="E1" s="90"/>
-      <c r="F1" s="90"/>
-      <c r="G1" s="91"/>
-    </row>
-    <row r="2" spans="2:7">
-      <c r="B2" s="94" t="s">
-        <v>171</v>
-      </c>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
-      <c r="E2" s="90"/>
-      <c r="F2" s="90"/>
-      <c r="G2" s="91"/>
+      <c r="C2" s="91"/>
+      <c r="D2" s="91"/>
+      <c r="E2" s="91"/>
+      <c r="F2" s="91"/>
+      <c r="G2" s="92"/>
     </row>
     <row r="3" spans="2:7">
       <c r="B3" s="3"/>
@@ -4506,7 +4505,7 @@
     </row>
     <row r="4" spans="2:7" ht="14.65" customHeight="1">
       <c r="B4" s="30" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C4" s="79">
         <v>-0.03</v>
@@ -4683,24 +4682,24 @@
       <c r="G11" s="3"/>
     </row>
     <row r="12" spans="2:7" ht="15.75" customHeight="1">
-      <c r="B12" s="89" t="s">
-        <v>173</v>
-      </c>
-      <c r="C12" s="90"/>
-      <c r="D12" s="90"/>
-      <c r="E12" s="90"/>
-      <c r="F12" s="90"/>
-      <c r="G12" s="91"/>
+      <c r="B12" s="90" t="s">
+        <v>172</v>
+      </c>
+      <c r="C12" s="91"/>
+      <c r="D12" s="91"/>
+      <c r="E12" s="91"/>
+      <c r="F12" s="91"/>
+      <c r="G12" s="92"/>
     </row>
     <row r="13" spans="2:7" ht="14.65" customHeight="1">
       <c r="B13" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C13" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D13" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -4708,7 +4707,7 @@
     </row>
     <row r="14" spans="2:7" ht="13.9" customHeight="1">
       <c r="B14" s="5" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C14" s="14">
         <f t="shared" ref="C14:C19" si="0">E5</f>
@@ -4724,7 +4723,7 @@
     </row>
     <row r="15" spans="2:7" ht="13.9" customHeight="1">
       <c r="B15" s="5" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C15" s="14">
         <f t="shared" si="0"/>
@@ -4740,7 +4739,7 @@
     </row>
     <row r="16" spans="2:7" ht="13.9" customHeight="1">
       <c r="B16" s="5" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C16" s="14">
         <f t="shared" si="0"/>
@@ -4756,7 +4755,7 @@
     </row>
     <row r="17" spans="2:7" ht="13.9" customHeight="1">
       <c r="B17" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C17" s="14">
         <f t="shared" si="0"/>
@@ -4772,7 +4771,7 @@
     </row>
     <row r="18" spans="2:7" ht="13.9" customHeight="1">
       <c r="B18" s="5" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C18" s="14">
         <f t="shared" si="0"/>
@@ -4788,7 +4787,7 @@
     </row>
     <row r="19" spans="2:7" ht="14.65" customHeight="1">
       <c r="B19" s="5" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C19" s="20">
         <f t="shared" si="0"/>
@@ -4811,24 +4810,24 @@
       <c r="G20" s="3"/>
     </row>
     <row r="21" spans="2:7" ht="15.75" customHeight="1">
-      <c r="B21" s="89" t="s">
-        <v>182</v>
-      </c>
-      <c r="C21" s="90"/>
-      <c r="D21" s="90"/>
-      <c r="E21" s="90"/>
-      <c r="F21" s="90"/>
-      <c r="G21" s="91"/>
+      <c r="B21" s="90" t="s">
+        <v>181</v>
+      </c>
+      <c r="C21" s="91"/>
+      <c r="D21" s="91"/>
+      <c r="E21" s="91"/>
+      <c r="F21" s="91"/>
+      <c r="G21" s="92"/>
     </row>
     <row r="22" spans="2:7" ht="14.65" customHeight="1">
       <c r="B22" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C22" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="D22" s="4" t="s">
         <v>174</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>175</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
@@ -4836,7 +4835,7 @@
     </row>
     <row r="23" spans="2:7" ht="13.9" customHeight="1">
       <c r="B23" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C23" s="14">
         <f>C10</f>
@@ -4852,7 +4851,7 @@
     </row>
     <row r="24" spans="2:7" ht="13.9" customHeight="1">
       <c r="B24" s="5" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C24" s="14">
         <f>D10</f>
@@ -4884,7 +4883,7 @@
     </row>
     <row r="26" spans="2:7" ht="13.9" customHeight="1">
       <c r="B26" s="5" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C26" s="14">
         <f>F10</f>
@@ -4931,40 +4930,40 @@
       <c r="G29" s="3"/>
     </row>
     <row r="30" spans="2:7" ht="14.65" customHeight="1">
-      <c r="B30" s="101" t="s">
+      <c r="B30" s="102" t="s">
+        <v>186</v>
+      </c>
+      <c r="C30" s="91"/>
+      <c r="D30" s="91"/>
+      <c r="E30" s="91"/>
+      <c r="F30" s="91"/>
+      <c r="G30" s="92"/>
+    </row>
+    <row r="31" spans="2:7" ht="34.049999999999997" customHeight="1">
+      <c r="B31" s="103" t="s">
         <v>187</v>
       </c>
-      <c r="C30" s="90"/>
-      <c r="D30" s="90"/>
-      <c r="E30" s="90"/>
-      <c r="F30" s="90"/>
-      <c r="G30" s="91"/>
-    </row>
-    <row r="31" spans="2:7" ht="34.049999999999997" customHeight="1">
-      <c r="B31" s="102" t="s">
-        <v>188</v>
-      </c>
-      <c r="C31" s="103"/>
-      <c r="D31" s="103"/>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103"/>
-      <c r="G31" s="104"/>
+      <c r="C31" s="104"/>
+      <c r="D31" s="104"/>
+      <c r="E31" s="104"/>
+      <c r="F31" s="104"/>
+      <c r="G31" s="105"/>
     </row>
     <row r="32" spans="2:7" ht="34.049999999999997" customHeight="1">
-      <c r="B32" s="105"/>
-      <c r="C32" s="88"/>
-      <c r="D32" s="88"/>
-      <c r="E32" s="88"/>
-      <c r="F32" s="88"/>
-      <c r="G32" s="106"/>
+      <c r="B32" s="106"/>
+      <c r="C32" s="89"/>
+      <c r="D32" s="89"/>
+      <c r="E32" s="89"/>
+      <c r="F32" s="89"/>
+      <c r="G32" s="107"/>
     </row>
     <row r="33" spans="2:7" ht="28.05" customHeight="1">
-      <c r="B33" s="107"/>
-      <c r="C33" s="108"/>
-      <c r="D33" s="108"/>
-      <c r="E33" s="108"/>
-      <c r="F33" s="108"/>
-      <c r="G33" s="109"/>
+      <c r="B33" s="108"/>
+      <c r="C33" s="109"/>
+      <c r="D33" s="109"/>
+      <c r="E33" s="109"/>
+      <c r="F33" s="109"/>
+      <c r="G33" s="110"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -4994,170 +4993,170 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:39" ht="28.05" customHeight="1">
-      <c r="A1" s="110" t="s">
-        <v>189</v>
-      </c>
-      <c r="B1" s="88"/>
-      <c r="C1" s="88"/>
-      <c r="D1" s="88"/>
-      <c r="E1" s="88"/>
-      <c r="F1" s="88"/>
-      <c r="G1" s="88"/>
-      <c r="H1" s="88"/>
-      <c r="I1" s="88"/>
-      <c r="J1" s="88"/>
-      <c r="K1" s="88"/>
-      <c r="L1" s="88"/>
-      <c r="M1" s="88"/>
-      <c r="N1" s="88"/>
-      <c r="O1" s="88"/>
-      <c r="P1" s="88"/>
-      <c r="Q1" s="88"/>
-      <c r="R1" s="88"/>
-      <c r="S1" s="88"/>
-      <c r="T1" s="88"/>
-      <c r="U1" s="88"/>
-      <c r="V1" s="88"/>
-      <c r="W1" s="88"/>
-      <c r="X1" s="88"/>
-      <c r="Y1" s="88"/>
-      <c r="Z1" s="88"/>
-      <c r="AA1" s="88"/>
-      <c r="AB1" s="88"/>
-      <c r="AC1" s="88"/>
-      <c r="AD1" s="88"/>
-      <c r="AE1" s="88"/>
-      <c r="AF1" s="88"/>
-      <c r="AG1" s="88"/>
-      <c r="AH1" s="88"/>
-      <c r="AI1" s="88"/>
-      <c r="AJ1" s="88"/>
-      <c r="AK1" s="88"/>
-      <c r="AL1" s="88"/>
-      <c r="AM1" s="88"/>
+      <c r="A1" s="111" t="s">
+        <v>188</v>
+      </c>
+      <c r="B1" s="89"/>
+      <c r="C1" s="89"/>
+      <c r="D1" s="89"/>
+      <c r="E1" s="89"/>
+      <c r="F1" s="89"/>
+      <c r="G1" s="89"/>
+      <c r="H1" s="89"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="89"/>
+      <c r="L1" s="89"/>
+      <c r="M1" s="89"/>
+      <c r="N1" s="89"/>
+      <c r="O1" s="89"/>
+      <c r="P1" s="89"/>
+      <c r="Q1" s="89"/>
+      <c r="R1" s="89"/>
+      <c r="S1" s="89"/>
+      <c r="T1" s="89"/>
+      <c r="U1" s="89"/>
+      <c r="V1" s="89"/>
+      <c r="W1" s="89"/>
+      <c r="X1" s="89"/>
+      <c r="Y1" s="89"/>
+      <c r="Z1" s="89"/>
+      <c r="AA1" s="89"/>
+      <c r="AB1" s="89"/>
+      <c r="AC1" s="89"/>
+      <c r="AD1" s="89"/>
+      <c r="AE1" s="89"/>
+      <c r="AF1" s="89"/>
+      <c r="AG1" s="89"/>
+      <c r="AH1" s="89"/>
+      <c r="AI1" s="89"/>
+      <c r="AJ1" s="89"/>
+      <c r="AK1" s="89"/>
+      <c r="AL1" s="89"/>
+      <c r="AM1" s="89"/>
     </row>
     <row r="3" spans="1:39" ht="24" customHeight="1">
       <c r="A3" s="85" t="s">
+        <v>189</v>
+      </c>
+      <c r="B3" s="85" t="s">
         <v>190</v>
       </c>
-      <c r="B3" s="85" t="s">
+      <c r="C3" s="85" t="s">
         <v>191</v>
       </c>
-      <c r="C3" s="85" t="s">
+      <c r="D3" s="85" t="s">
         <v>192</v>
       </c>
-      <c r="D3" s="85" t="s">
+      <c r="E3" s="85" t="s">
         <v>193</v>
       </c>
-      <c r="E3" s="85" t="s">
+      <c r="F3" s="85" t="s">
         <v>194</v>
       </c>
-      <c r="F3" s="85" t="s">
+      <c r="G3" s="85" t="s">
         <v>195</v>
       </c>
-      <c r="G3" s="85" t="s">
+      <c r="H3" s="85" t="s">
         <v>196</v>
       </c>
-      <c r="H3" s="85" t="s">
+      <c r="I3" s="85" t="s">
         <v>197</v>
       </c>
-      <c r="I3" s="85" t="s">
+      <c r="J3" s="85" t="s">
         <v>198</v>
       </c>
-      <c r="J3" s="85" t="s">
+      <c r="K3" s="85" t="s">
         <v>199</v>
       </c>
-      <c r="K3" s="85" t="s">
+      <c r="L3" s="85" t="s">
         <v>200</v>
       </c>
-      <c r="L3" s="85" t="s">
+      <c r="M3" s="85" t="s">
         <v>201</v>
       </c>
-      <c r="M3" s="85" t="s">
+      <c r="N3" s="85" t="s">
         <v>202</v>
       </c>
-      <c r="N3" s="85" t="s">
+      <c r="O3" s="85" t="s">
         <v>203</v>
       </c>
-      <c r="O3" s="85" t="s">
+      <c r="P3" s="85" t="s">
         <v>204</v>
       </c>
-      <c r="P3" s="85" t="s">
+      <c r="Q3" s="85" t="s">
         <v>205</v>
       </c>
-      <c r="Q3" s="85" t="s">
+      <c r="R3" s="85" t="s">
         <v>206</v>
       </c>
-      <c r="R3" s="85" t="s">
+      <c r="S3" s="85" t="s">
         <v>207</v>
       </c>
-      <c r="S3" s="85" t="s">
+      <c r="T3" s="85" t="s">
         <v>208</v>
       </c>
-      <c r="T3" s="85" t="s">
+      <c r="U3" s="85" t="s">
         <v>209</v>
       </c>
-      <c r="U3" s="85" t="s">
+      <c r="V3" s="85" t="s">
         <v>210</v>
       </c>
-      <c r="V3" s="85" t="s">
+      <c r="W3" s="85" t="s">
         <v>211</v>
       </c>
-      <c r="W3" s="85" t="s">
+      <c r="X3" s="85" t="s">
         <v>212</v>
       </c>
-      <c r="X3" s="85" t="s">
+      <c r="Y3" s="85" t="s">
         <v>213</v>
       </c>
-      <c r="Y3" s="85" t="s">
+      <c r="Z3" s="85" t="s">
         <v>214</v>
       </c>
-      <c r="Z3" s="85" t="s">
+      <c r="AA3" s="85" t="s">
         <v>215</v>
       </c>
-      <c r="AA3" s="85" t="s">
+      <c r="AB3" s="85" t="s">
         <v>216</v>
       </c>
-      <c r="AB3" s="85" t="s">
+      <c r="AC3" s="85" t="s">
         <v>217</v>
       </c>
-      <c r="AC3" s="85" t="s">
+      <c r="AD3" s="85" t="s">
         <v>218</v>
       </c>
-      <c r="AD3" s="85" t="s">
+      <c r="AE3" s="85" t="s">
         <v>219</v>
       </c>
-      <c r="AE3" s="85" t="s">
+      <c r="AF3" s="85" t="s">
         <v>220</v>
       </c>
-      <c r="AF3" s="85" t="s">
+      <c r="AG3" s="85" t="s">
         <v>221</v>
       </c>
-      <c r="AG3" s="85" t="s">
+      <c r="AH3" s="85" t="s">
         <v>222</v>
       </c>
-      <c r="AH3" s="85" t="s">
+      <c r="AI3" s="85" t="s">
         <v>223</v>
       </c>
-      <c r="AI3" s="85" t="s">
+      <c r="AJ3" s="85" t="s">
         <v>224</v>
       </c>
-      <c r="AJ3" s="85" t="s">
+      <c r="AK3" s="85" t="s">
         <v>225</v>
       </c>
-      <c r="AK3" s="85" t="s">
+      <c r="AL3" s="85" t="s">
         <v>226</v>
       </c>
-      <c r="AL3" s="85" t="s">
+      <c r="AM3" s="85" t="s">
         <v>227</v>
-      </c>
-      <c r="AM3" s="85" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="4" spans="1:39">
       <c r="A4" s="82" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B4" s="83">
         <v>0.7</v>
@@ -5312,7 +5311,7 @@
     </row>
     <row r="5" spans="1:39">
       <c r="A5" s="82" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B5" s="83">
         <v>0.7</v>
@@ -5467,7 +5466,7 @@
     </row>
     <row r="6" spans="1:39">
       <c r="A6" s="82" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B6" s="83">
         <v>0.7</v>
@@ -5622,7 +5621,7 @@
     </row>
     <row r="7" spans="1:39">
       <c r="A7" s="82" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B7" s="83">
         <v>0.7</v>
@@ -5777,7 +5776,7 @@
     </row>
     <row r="8" spans="1:39">
       <c r="A8" s="82" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B8" s="83">
         <v>0.7</v>
@@ -5932,7 +5931,7 @@
     </row>
     <row r="9" spans="1:39">
       <c r="A9" s="82" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B9" s="83">
         <v>0.75</v>
@@ -6087,7 +6086,7 @@
     </row>
     <row r="10" spans="1:39">
       <c r="A10" s="82" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B10" s="83">
         <v>0.75</v>
@@ -6242,7 +6241,7 @@
     </row>
     <row r="11" spans="1:39">
       <c r="A11" s="82" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B11" s="83">
         <v>0.75</v>
@@ -6397,7 +6396,7 @@
     </row>
     <row r="12" spans="1:39">
       <c r="A12" s="82" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B12" s="83">
         <v>0.75</v>
@@ -6552,7 +6551,7 @@
     </row>
     <row r="13" spans="1:39">
       <c r="A13" s="82" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B13" s="83">
         <v>0.75</v>
@@ -6707,7 +6706,7 @@
     </row>
     <row r="14" spans="1:39">
       <c r="A14" s="82" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B14" s="83">
         <v>0.8</v>
@@ -6862,7 +6861,7 @@
     </row>
     <row r="15" spans="1:39">
       <c r="A15" s="82" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B15" s="83">
         <v>0.8</v>
@@ -7017,7 +7016,7 @@
     </row>
     <row r="16" spans="1:39">
       <c r="A16" s="82" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B16" s="83">
         <v>0.8</v>
@@ -7172,7 +7171,7 @@
     </row>
     <row r="17" spans="1:39">
       <c r="A17" s="82" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B17" s="83">
         <v>0.8</v>
@@ -7327,7 +7326,7 @@
     </row>
     <row r="18" spans="1:39">
       <c r="A18" s="82" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B18" s="83">
         <v>0.8</v>
@@ -7482,7 +7481,7 @@
     </row>
     <row r="19" spans="1:39">
       <c r="A19" s="82" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B19" s="83">
         <v>0.85</v>
@@ -7637,7 +7636,7 @@
     </row>
     <row r="20" spans="1:39">
       <c r="A20" s="82" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B20" s="83">
         <v>0.85</v>
@@ -7792,7 +7791,7 @@
     </row>
     <row r="21" spans="1:39">
       <c r="A21" s="82" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B21" s="83">
         <v>0.85</v>
@@ -7947,7 +7946,7 @@
     </row>
     <row r="22" spans="1:39">
       <c r="A22" s="82" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B22" s="83">
         <v>0.85</v>
@@ -8102,7 +8101,7 @@
     </row>
     <row r="23" spans="1:39">
       <c r="A23" s="82" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B23" s="83">
         <v>0.85</v>
@@ -8257,7 +8256,7 @@
     </row>
     <row r="24" spans="1:39">
       <c r="A24" s="82" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="B24" s="83">
         <v>0.9</v>
@@ -8412,7 +8411,7 @@
     </row>
     <row r="25" spans="1:39">
       <c r="A25" s="82" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B25" s="83">
         <v>0.9</v>
@@ -8567,7 +8566,7 @@
     </row>
     <row r="26" spans="1:39">
       <c r="A26" s="82" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="B26" s="83">
         <v>0.9</v>
@@ -8722,7 +8721,7 @@
     </row>
     <row r="27" spans="1:39">
       <c r="A27" s="82" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B27" s="83">
         <v>0.9</v>
@@ -8877,7 +8876,7 @@
     </row>
     <row r="28" spans="1:39">
       <c r="A28" s="82" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B28" s="83">
         <v>0.9</v>
@@ -9032,7 +9031,7 @@
     </row>
     <row r="29" spans="1:39">
       <c r="A29" s="82" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="B29" s="83">
         <v>0.95</v>
@@ -9187,7 +9186,7 @@
     </row>
     <row r="30" spans="1:39">
       <c r="A30" s="82" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="B30" s="83">
         <v>0.95</v>
@@ -9342,7 +9341,7 @@
     </row>
     <row r="31" spans="1:39">
       <c r="A31" s="82" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="B31" s="83">
         <v>0.95</v>
@@ -9497,7 +9496,7 @@
     </row>
     <row r="32" spans="1:39">
       <c r="A32" s="82" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="B32" s="83">
         <v>0.95</v>
@@ -9652,7 +9651,7 @@
     </row>
     <row r="33" spans="1:39">
       <c r="A33" s="82" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="B33" s="83">
         <v>0.95</v>
@@ -9811,6 +9810,6 @@
   </mergeCells>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.2" right="0.2" top="0.3" bottom="0.3" header="0.1" footer="0.1"/>
-  <pageSetup paperSize="9" fitToWidth="3" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="78" fitToWidth="3" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>